<commit_message>
feat(autres-flux): paramétrage affectation + références UUID
- Ajout colonnes 'Affectation type' / 'Affectation cible (UUID)' / 'Affectation cible (nom)'
  sur SERVICE_ACHAT et NOUVELLES_ETAPES (à remplir sur la ligne N°=1 de chaque sous-processus)
- Ajout colonne ID_sous_processus + Sous-processus dans NOUVELLES_ETAPES
- Nouveau snapshot _refs-snapshot.json : 102 profils + 62 départements
- Onglet PROFILES_REFERENCE + DEPARTMENTS_REFERENCE + ASSIGNMENT_TYPES (cheat-sheet)
- Onglet ETATS_PAR_FLUX étendu avec colonne 'Catégorie' macro (6 valeurs)
- LISEZ-MOI mis à jour avec les nouvelles règles d'affectation

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AUTRES_FLUX_parametrage.xlsx
+++ b/AUTRES_FLUX_parametrage.xlsx
@@ -6,8 +6,11 @@
     <sheet name="SERVICE_ACHAT" sheetId="1" r:id="rId1"/>
     <sheet name="NOUVELLES_ETAPES" sheetId="2" r:id="rId2"/>
     <sheet name="PROCESS_REFERENCE" sheetId="3" r:id="rId3"/>
-    <sheet name="ETATS_PAR_FLUX" sheetId="4" r:id="rId4"/>
-    <sheet name="LISEZ-MOI" sheetId="5" r:id="rId5"/>
+    <sheet name="PROFILES_REFERENCE" sheetId="4" r:id="rId4"/>
+    <sheet name="DEPARTMENTS_REFERENCE" sheetId="5" r:id="rId5"/>
+    <sheet name="ASSIGNMENT_TYPES" sheetId="6" r:id="rId6"/>
+    <sheet name="ETATS_PAR_FLUX" sheetId="7" r:id="rId7"/>
+    <sheet name="LISEZ-MOI" sheetId="8" r:id="rId8"/>
   </sheets>
 </workbook>
 </file>
@@ -401,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:Q4"/>
   <cols>
     <col min="1" max="1" width="38.83203125" customWidth="1"/>
     <col min="2" max="2" width="38.83203125" customWidth="1"/>
@@ -409,14 +412,17 @@
     <col min="4" max="4" width="5.83203125" customWidth="1"/>
     <col min="5" max="5" width="36.83203125" customWidth="1"/>
     <col min="6" max="6" width="11.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="30.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="22.83203125" customWidth="1"/>
-    <col min="12" max="12" width="18.83203125" customWidth="1"/>
-    <col min="13" max="13" width="22.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="20.83203125" customWidth="1"/>
+    <col min="11" max="11" width="38.83203125" customWidth="1"/>
+    <col min="12" max="12" width="30.83203125" customWidth="1"/>
+    <col min="13" max="13" width="18.83203125" customWidth="1"/>
+    <col min="14" max="14" width="18.83203125" customWidth="1"/>
+    <col min="15" max="15" width="22.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -448,18 +454,27 @@
         <v>Délai après précédente (j)</v>
       </c>
       <c r="J1" t="str">
+        <v>Affectation type</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Affectation cible (UUID)</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Affectation cible (nom)</v>
+      </c>
+      <c r="M1" t="str">
         <v>Validation N1</v>
       </c>
-      <c r="K1" t="str">
+      <c r="N1" t="str">
         <v>Valideur N1</v>
       </c>
-      <c r="L1" t="str">
+      <c r="O1" t="str">
         <v>Validation N2</v>
       </c>
-      <c r="M1" t="str">
+      <c r="P1" t="str">
         <v>Valideur N2</v>
       </c>
-      <c r="N1" t="str">
+      <c r="Q1" t="str">
         <v>État en sortie</v>
       </c>
     </row>
@@ -492,18 +507,27 @@
         <v>0</v>
       </c>
       <c r="J2" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
         <v>aucune</v>
       </c>
-      <c r="K2" t="str">
-        <v/>
-      </c>
-      <c r="L2" t="str">
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
         <v>aucune</v>
       </c>
-      <c r="M2" t="str">
-        <v/>
-      </c>
-      <c r="N2" t="str">
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
         <v/>
       </c>
     </row>
@@ -536,18 +560,27 @@
         <v>0</v>
       </c>
       <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
         <v>aucune</v>
       </c>
-      <c r="K3" t="str">
-        <v/>
-      </c>
-      <c r="L3" t="str">
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
         <v>aucune</v>
       </c>
-      <c r="M3" t="str">
-        <v/>
-      </c>
-      <c r="N3" t="str">
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
         <v/>
       </c>
     </row>
@@ -580,45 +613,59 @@
         <v>0</v>
       </c>
       <c r="J4" t="str">
+        <v>fixed_user</v>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
         <v>aucune</v>
       </c>
-      <c r="K4" t="str">
-        <v/>
-      </c>
-      <c r="L4" t="str">
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
         <v>aucune</v>
       </c>
-      <c r="M4" t="str">
-        <v/>
-      </c>
-      <c r="N4" t="str">
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:R9"/>
   <cols>
     <col min="1" max="1" width="38.83203125" customWidth="1"/>
     <col min="2" max="2" width="42.83203125" customWidth="1"/>
-    <col min="3" max="3" width="5.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="38.83203125" customWidth="1"/>
+    <col min="4" max="4" width="42.83203125" customWidth="1"/>
+    <col min="5" max="5" width="5.83203125" customWidth="1"/>
+    <col min="6" max="6" width="36.83203125" customWidth="1"/>
+    <col min="7" max="7" width="11.83203125" customWidth="1"/>
     <col min="8" max="8" width="18.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="22.83203125" customWidth="1"/>
-    <col min="11" max="11" width="18.83203125" customWidth="1"/>
-    <col min="12" max="12" width="22.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="20.83203125" customWidth="1"/>
+    <col min="10" max="10" width="24.83203125" customWidth="1"/>
+    <col min="11" max="11" width="20.83203125" customWidth="1"/>
+    <col min="12" max="12" width="38.83203125" customWidth="1"/>
+    <col min="13" max="13" width="30.83203125" customWidth="1"/>
+    <col min="14" max="14" width="18.83203125" customWidth="1"/>
+    <col min="15" max="15" width="18.83203125" customWidth="1"/>
+    <col min="16" max="16" width="22.83203125" customWidth="1"/>
+    <col min="17" max="17" width="18.83203125" customWidth="1"/>
+    <col min="18" max="18" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -629,36 +676,51 @@
         <v>Processus</v>
       </c>
       <c r="C1" t="str">
+        <v>ID_sous_processus</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Sous-processus</v>
+      </c>
+      <c r="E1" t="str">
         <v>N°</v>
       </c>
-      <c r="D1" t="str">
+      <c r="F1" t="str">
         <v>Étape</v>
       </c>
-      <c r="E1" t="str">
+      <c r="G1" t="str">
         <v>Durée (j)</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>Démarrage</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>Dépend de (étape n°)</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>Délai après précédente (j)</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
+        <v>Affectation type</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Affectation cible (UUID)</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Affectation cible (nom)</v>
+      </c>
+      <c r="N1" t="str">
         <v>Validation N1</v>
       </c>
-      <c r="J1" t="str">
+      <c r="O1" t="str">
         <v>Valideur N1</v>
       </c>
-      <c r="K1" t="str">
+      <c r="P1" t="str">
         <v>Validation N2</v>
       </c>
-      <c r="L1" t="str">
+      <c r="Q1" t="str">
         <v>Valideur N2</v>
       </c>
-      <c r="M1" t="str">
+      <c r="R1" t="str">
         <v>État en sortie</v>
       </c>
     </row>
@@ -669,8 +731,8 @@
       <c r="B2" t="str">
         <v/>
       </c>
-      <c r="C2">
-        <v>1</v>
+      <c r="C2" t="str">
+        <v/>
       </c>
       <c r="D2" t="str">
         <v/>
@@ -679,27 +741,42 @@
         <v>1</v>
       </c>
       <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2" t="str">
         <v>parallele</v>
       </c>
-      <c r="G2" t="str">
-        <v/>
-      </c>
-      <c r="H2">
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2">
         <v>0</v>
       </c>
-      <c r="I2" t="str">
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
         <v>aucune</v>
       </c>
-      <c r="J2" t="str">
-        <v/>
-      </c>
-      <c r="K2" t="str">
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
         <v>aucune</v>
       </c>
-      <c r="L2" t="str">
-        <v/>
-      </c>
-      <c r="M2" t="str">
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+      <c r="R2" t="str">
         <v/>
       </c>
     </row>
@@ -710,8 +787,8 @@
       <c r="B3" t="str">
         <v/>
       </c>
-      <c r="C3">
-        <v>1</v>
+      <c r="C3" t="str">
+        <v/>
       </c>
       <c r="D3" t="str">
         <v/>
@@ -720,27 +797,42 @@
         <v>1</v>
       </c>
       <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3" t="str">
         <v>parallele</v>
       </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3">
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3">
         <v>0</v>
       </c>
-      <c r="I3" t="str">
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
         <v>aucune</v>
       </c>
-      <c r="J3" t="str">
-        <v/>
-      </c>
-      <c r="K3" t="str">
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
         <v>aucune</v>
       </c>
-      <c r="L3" t="str">
-        <v/>
-      </c>
-      <c r="M3" t="str">
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
         <v/>
       </c>
     </row>
@@ -751,8 +843,8 @@
       <c r="B4" t="str">
         <v/>
       </c>
-      <c r="C4">
-        <v>1</v>
+      <c r="C4" t="str">
+        <v/>
       </c>
       <c r="D4" t="str">
         <v/>
@@ -761,27 +853,42 @@
         <v>1</v>
       </c>
       <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4" t="str">
         <v>parallele</v>
       </c>
-      <c r="G4" t="str">
-        <v/>
-      </c>
-      <c r="H4">
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4">
         <v>0</v>
       </c>
-      <c r="I4" t="str">
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
         <v>aucune</v>
       </c>
-      <c r="J4" t="str">
-        <v/>
-      </c>
-      <c r="K4" t="str">
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
         <v>aucune</v>
       </c>
-      <c r="L4" t="str">
-        <v/>
-      </c>
-      <c r="M4" t="str">
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
         <v/>
       </c>
     </row>
@@ -792,8 +899,8 @@
       <c r="B5" t="str">
         <v/>
       </c>
-      <c r="C5">
-        <v>1</v>
+      <c r="C5" t="str">
+        <v/>
       </c>
       <c r="D5" t="str">
         <v/>
@@ -802,27 +909,42 @@
         <v>1</v>
       </c>
       <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5" t="str">
         <v>parallele</v>
       </c>
-      <c r="G5" t="str">
-        <v/>
-      </c>
-      <c r="H5">
+      <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5">
         <v>0</v>
       </c>
-      <c r="I5" t="str">
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
         <v>aucune</v>
       </c>
-      <c r="J5" t="str">
-        <v/>
-      </c>
-      <c r="K5" t="str">
+      <c r="O5" t="str">
+        <v/>
+      </c>
+      <c r="P5" t="str">
         <v>aucune</v>
       </c>
-      <c r="L5" t="str">
-        <v/>
-      </c>
-      <c r="M5" t="str">
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
         <v/>
       </c>
     </row>
@@ -833,8 +955,8 @@
       <c r="B6" t="str">
         <v/>
       </c>
-      <c r="C6">
-        <v>1</v>
+      <c r="C6" t="str">
+        <v/>
       </c>
       <c r="D6" t="str">
         <v/>
@@ -843,33 +965,216 @@
         <v>1</v>
       </c>
       <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6" t="str">
         <v>parallele</v>
       </c>
-      <c r="G6" t="str">
-        <v/>
-      </c>
-      <c r="H6">
+      <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6">
         <v>0</v>
       </c>
-      <c r="I6" t="str">
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
         <v>aucune</v>
       </c>
-      <c r="J6" t="str">
-        <v/>
-      </c>
-      <c r="K6" t="str">
+      <c r="O6" t="str">
+        <v/>
+      </c>
+      <c r="P6" t="str">
         <v>aucune</v>
       </c>
-      <c r="L6" t="str">
-        <v/>
-      </c>
-      <c r="M6" t="str">
+      <c r="Q6" t="str">
+        <v/>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7" t="str">
+        <v>parallele</v>
+      </c>
+      <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7" t="str">
+        <v/>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v>aucune</v>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+      <c r="P7" t="str">
+        <v>aucune</v>
+      </c>
+      <c r="Q7" t="str">
+        <v/>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v/>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8" t="str">
+        <v>parallele</v>
+      </c>
+      <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v>aucune</v>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+      <c r="P8" t="str">
+        <v>aucune</v>
+      </c>
+      <c r="Q8" t="str">
+        <v/>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9" t="str">
+        <v>parallele</v>
+      </c>
+      <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9" t="str">
+        <v/>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v>aucune</v>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+      <c r="P9" t="str">
+        <v>aucune</v>
+      </c>
+      <c r="Q9" t="str">
+        <v/>
+      </c>
+      <c r="R9" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1059,7 +1364,2064 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:D103"/>
+  <cols>
+    <col min="1" max="1" width="40.83203125" customWidth="1"/>
+    <col min="2" max="2" width="32.83203125" customWidth="1"/>
+    <col min="3" max="3" width="48.83203125" customWidth="1"/>
+    <col min="4" max="4" width="28.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>UUID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Nom</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Fonction</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Département</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>feeb2a94-64fc-4527-8970-5eba19530844</v>
+      </c>
+      <c r="B2" t="str">
+        <v>AMANOUNE Karim</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Stagiaire Analyste financier</v>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>4c76ad87-031a-4313-a4ce-380380d4d7be</v>
+      </c>
+      <c r="B3" t="str">
+        <v>ANTHONEY Noemie</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Gestionnaire Administratif et Comptable</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Comptabilité</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>bb9c06f6-910b-4d5d-afb0-d31e1d90c77d</v>
+      </c>
+      <c r="B4" t="str">
+        <v>ANTZ Sylvain</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Coordinateur(rice) Maintenance</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Maintenance</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>7c6c7ec0-eb37-47f5-8464-e6fb78c05fb7</v>
+      </c>
+      <c r="B5" t="str">
+        <v>AUBREE Maxime</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Technico-Commercial</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Commercial Sycomore</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>d088d312-b68c-4456-ad10-55c94c05cd0d</v>
+      </c>
+      <c r="B6" t="str">
+        <v>AUNILLON Julien</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Ingénieur(e) d'Etudes</v>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>1a8187b1-0d73-45ea-b5fe-a1b9c1d93a0a</v>
+      </c>
+      <c r="B7" t="str">
+        <v>BAFFOU Alexandre</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Responsable Achats et logistique</v>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>963c2ca8-1b43-4d18-a8ad-3c09cccb16ad</v>
+      </c>
+      <c r="B8" t="str">
+        <v>BAIDOSHVILI Nikolozi</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Chef de projet SIG</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>8926222c-b09f-4bf4-bb50-a37ba5dd896c</v>
+      </c>
+      <c r="B9" t="str">
+        <v>BARATON Alain</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Chef de Projet développement</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Montage de projet France</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>d4f8b0b6-42b1-43aa-8491-c86734ee2ae2</v>
+      </c>
+      <c r="B10" t="str">
+        <v>BEREHOUC Romain</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Directeur(rice) NASKEO</v>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>96b5ac13-fbb0-417f-bc68-291155dc61ef</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Berthet Clément</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Chargé(e) de Développement commercial</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>ef3805a3-b3c8-40a4-ab48-811a9bc814e3</v>
+      </c>
+      <c r="B12" t="str">
+        <v>BERTIN Charlotte</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Ingénieur(e) d'Etudes d'exploitation</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Execution Naskeo</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>81750c79-efb6-48e2-8788-0ec9a6f13b68</v>
+      </c>
+      <c r="B13" t="str">
+        <v>BERTRAND Valentin</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Responsable des Systèmes d'information</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>011e0abd-c763-42e4-b4ca-d0d3e7384396</v>
+      </c>
+      <c r="B14" t="str">
+        <v>BEUTIER Corinne</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Directeur(rice) Administratif et Financier</v>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>5b16e383-aef8-4bd2-98c8-dfe47b4a0a9b</v>
+      </c>
+      <c r="B15" t="str">
+        <v>BIGOT Simon</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Responsable d'Etudes d'exploitation</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Execution Naskeo</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>b4745401-7cea-4400-a865-2ce7289d3989</v>
+      </c>
+      <c r="B16" t="str">
+        <v>BOCQUILLON Leila</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Chef de Projet développement</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Montage de projet France</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>4b64e971-eaf8-4178-a184-230e5ee1b975</v>
+      </c>
+      <c r="B17" t="str">
+        <v>BOLO Camille</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Responsable des Ressources Humaines</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Ressources Humaines</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>e4822dc4-362a-4ccc-bfda-1dae219774b3</v>
+      </c>
+      <c r="B18" t="str">
+        <v>BOUR Grégoire</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Directeur du développement international</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Montage de projet Int.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>f97c5977-af5f-4640-a589-961884915c29</v>
+      </c>
+      <c r="B19" t="str">
+        <v>BOUVRON Kevin</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Ingénieur(e) Réalisation</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Réalisation</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>a56e41e4-0774-4488-8143-df3f3e3ae32a</v>
+      </c>
+      <c r="B20" t="str">
+        <v>CHABALIER Cédric</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Responsable de Site</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Les 3 dômes</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>37408a59-e076-48c6-9d49-08e4977d130a</v>
+      </c>
+      <c r="B21" t="str">
+        <v>CHAGHOURI Muriel</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Ingénieur(e) R&amp;D</v>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>e8d5e5f4-3cd3-4f6d-839f-189341727095</v>
+      </c>
+      <c r="B22" t="str">
+        <v>CHASTANG Céline</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Contrôleur(se) de Gestion</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Contrôle de Gestion</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>455b3daf-22a3-4591-951f-7134b258a110</v>
+      </c>
+      <c r="B23" t="str">
+        <v>CHAUMET Astrid</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Analyste Financière M&amp;A</v>
+      </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>f326eeb1-3d92-45e5-a957-8e02bda84115</v>
+      </c>
+      <c r="B24" t="str">
+        <v>CLERMONT SOPHIE</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Directrice du Développement de Keon</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Montage de projet France</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>4c1826c8-ee97-43a2-91f6-a300d4d88cab</v>
+      </c>
+      <c r="B25" t="str">
+        <v>CORRIER Naylor</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Gestionnaire administrative et comptable confirmée</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Comptabilité</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>6343b0a6-28ca-46ab-8c28-f1f3c57d8207</v>
+      </c>
+      <c r="B26" t="str">
+        <v>COSTAL Virgile</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Responsable de Conception</v>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>f46a0644-e97f-4120-8f60-36bc63f4c249</v>
+      </c>
+      <c r="B27" t="str">
+        <v>COUZY Sébastien</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Responsable des Affaires juridiques</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Juridique</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>92f03d5a-a386-4eba-99e5-0ca6d3c414c7</v>
+      </c>
+      <c r="B28" t="str">
+        <v>CRAIPEAU Hugo</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Ingénieur(e) Réalisation</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Réalisation</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>955c8485-5784-46c9-a8ca-f8c14347fa6f</v>
+      </c>
+      <c r="B29" t="str">
+        <v>CROSET Romain</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Chef de Site</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Gatinais Déconditionnement</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>b1502948-97c5-4ddb-b3a5-dbc6484f0933</v>
+      </c>
+      <c r="B30" t="str">
+        <v>DA FONSECA Aurore</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Chef de Projet développement</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Montage de projet France</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>174f0771-845a-4e30-81fa-5e45c65d78eb</v>
+      </c>
+      <c r="B31" t="str">
+        <v>DAVID Marie</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Chef de Projet développement</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Montage de projet France</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>66a6a1cb-19a4-4aea-90f2-011a6045e24c</v>
+      </c>
+      <c r="B32" t="str">
+        <v>DE LA GOURNERIE Paul</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Ingénieur(e) Réalisation</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Réalisation</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>ee676b11-624b-4c6a-8cb1-3e19523a59cc</v>
+      </c>
+      <c r="B33" t="str">
+        <v>DELHOMME Damien</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Chef de projets développement Canada</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Montage de projet Int.</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>28d2525e-9ccc-4b13-904d-ff0dcaab4b46</v>
+      </c>
+      <c r="B34" t="str">
+        <v>DEMIRDJI Shnorh</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Gestionnaire Administratif et Comptable</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Comptabilité</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>e3ea4f4a-d65b-40c8-8eb3-fa1f96990b1a</v>
+      </c>
+      <c r="B35" t="str">
+        <v>DIANTETELA Myriam</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Chargé(e) des Ressources Humaines</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Ressources Humaines</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>b2e144be-1c11-4613-ab83-ebb385eba859</v>
+      </c>
+      <c r="B36" t="str">
+        <v>DURAMPART Maxime</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Ingénieur d'études d'exécutions</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Mise en service</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>f3e0b701-c15b-4f5d-9674-73cc7992e9b8</v>
+      </c>
+      <c r="B37" t="str">
+        <v>FAUTRAS Damien</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Gestionnaire Administratif et Comptable</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Comptabilité</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>45e2d4a0-8446-4d03-8459-89b0cf432982</v>
+      </c>
+      <c r="B38" t="str">
+        <v>FISGATIVA Henry</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Coordinateur(rice) R&amp;D</v>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>bbd9484c-cb96-4b4e-82ef-b88d556254f2</v>
+      </c>
+      <c r="B39" t="str">
+        <v>FOLTZENLOGEL Patrick</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Directeur(rice) Général Délégué</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Direction Générale</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>5e2b4969-9b04-4dbc-af5d-8bf9137dd57b</v>
+      </c>
+      <c r="B40" t="str">
+        <v>FOULONNEAU Amaury</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Ingénieur(e) Exploitation</v>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>8794eb1a-93d2-4250-a3e6-a36bc14c17ab</v>
+      </c>
+      <c r="B41" t="str">
+        <v>GARDONI Jean-Yves</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Expert Méthanisation</v>
+      </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>5a8b682a-8e2a-41b7-bb25-bbae32a0ea1d</v>
+      </c>
+      <c r="B42" t="str">
+        <v>GHISLOTTI-BONALDI Marco</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Business Developer international</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Montage de projet Int.</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>33d1e9ba-86d8-4086-9cdc-2b819ea9777b</v>
+      </c>
+      <c r="B43" t="str">
+        <v>GILLET Stephane</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Responsable des Acquisitions</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Acquisitions</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>00895a79-675e-41ce-a31d-331538880b66</v>
+      </c>
+      <c r="B44" t="str">
+        <v>GREGOIRE Camille</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Ingénieur(e) d'Etudes d'exploitation</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Execution Naskeo</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>642a531d-3a2e-4252-a0ba-785b584d5add</v>
+      </c>
+      <c r="B45" t="str">
+        <v>GROSBOST Magali</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Ingénieur(e) d'Etudes</v>
+      </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>18755c38-0673-41a0-8de8-db6fa7de3d35</v>
+      </c>
+      <c r="B46" t="str">
+        <v>GROSSIN Axel</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Ingénieur(e) d'Etudes</v>
+      </c>
+      <c r="D46" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>92617bd1-c6f8-412f-9593-d71e7088a712</v>
+      </c>
+      <c r="B47" t="str">
+        <v>GUILBAUD Paul</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Responsable projets – Conception et Exploitation et Responsable des partenariats</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Acquisitions</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>947d3326-ef79-4c4c-9e48-0778a41e440c</v>
+      </c>
+      <c r="B48" t="str">
+        <v>HAUMONT François</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Directeur(rice) Commercial</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Direction Commerciale</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>e94606e3-2023-44d3-88ba-85b1f294ba24</v>
+      </c>
+      <c r="B49" t="str">
+        <v>HOFMAN Adrienne</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Ingénieur(e) d'Etudes</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Reglementation</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>13b61d6d-4db4-4231-b8fc-4593ae747338</v>
+      </c>
+      <c r="B50" t="str">
+        <v>HULINE Emilie</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Coordinateur(rice) Laboratoire</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Laboratoire</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>eb1ca217-911a-4802-8bae-274a54445ff1</v>
+      </c>
+      <c r="B51" t="str">
+        <v>JACQ Gwenaelle</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Responsable Biomasse et approvisionnement déchets</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Approvisionnement</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>8acf06a1-7968-4e2b-85c8-687c2bba4ceb</v>
+      </c>
+      <c r="B52" t="str">
+        <v>JOLIVEL Anael</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Ingénieur(e) Maître d'Ouvrage</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Maîtrise d'ouvrage</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>5abd7e99-48e4-4d39-b3e0-84be21fcb989</v>
+      </c>
+      <c r="B53" t="str">
+        <v>KABECHE Lyza</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Automaticien(ne)</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Automatisme</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>791009d8-65f2-40ac-be5f-d0c468df1480</v>
+      </c>
+      <c r="B54" t="str">
+        <v>KABORE Audrey</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Responsable des Ressources Humaines Adjointe</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Ressources Humaines</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>377c3f30-8ace-41dd-9ffe-de1865f7451d</v>
+      </c>
+      <c r="B55" t="str">
+        <v>KHOUAS Nicolas</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Conducteur de Travaux génie civil</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Génie Civil</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>90ffb29c-4887-480d-b075-9b66a6c4dd26</v>
+      </c>
+      <c r="B56" t="str">
+        <v>KOCET Nicolas</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Responsable Réalisation</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Réalisation</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>ad215d38-063a-4af5-9a2d-8a8941e59f3d</v>
+      </c>
+      <c r="B57" t="str">
+        <v>KOZERAWSKI Pascal</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Responsable Régional Ouest</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Pole Exploitation Nord-Ouest</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>58e64899-0f72-4cd1-a553-f45ebdb1a771</v>
+      </c>
+      <c r="B58" t="str">
+        <v>L'HERIAU Germain</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Responsable Commercial</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Commercial Naskeo</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>00e1476d-46e3-4a28-aaa5-63c0a9498b75</v>
+      </c>
+      <c r="B59" t="str">
+        <v>LABRUNIE Pierre</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Responsable Mise en service</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Mise en service</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>5879a4e5-17a6-46ce-b94f-d4aaa0dd53fc</v>
+      </c>
+      <c r="B60" t="str">
+        <v>LANTRAN Erwan</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Dessinateur(rice) Projeteur</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Dessin</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>baf15ab5-781c-4693-b697-e4a4f3de02bb</v>
+      </c>
+      <c r="B61" t="str">
+        <v>LAPEYRE Paul</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Magasinier</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Logistique</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>f23cd2a4-6f9c-431e-b095-0f2f90a04698</v>
+      </c>
+      <c r="B62" t="str">
+        <v>LAUREILLARD Alane</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Chargé(e) d'Affaires Grand Est</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Approvisionnement</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>4f398578-6600-464a-bb4c-9a5349fc2322</v>
+      </c>
+      <c r="B63" t="str">
+        <v>LEBRUN Evan</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Responsable des Partenariats</v>
+      </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>3aceec71-c601-40d1-b3ea-fcd3938774c3</v>
+      </c>
+      <c r="B64" t="str">
+        <v>LEFEBVRE Aurélien</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Responsable de Projet Canada</v>
+      </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>61208480-642c-4584-b29a-8c538e83d45c</v>
+      </c>
+      <c r="B65" t="str">
+        <v>LELAIDIER Aline</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Responsable de site</v>
+      </c>
+      <c r="D65" t="str">
+        <v>Biogaz de Bel Air</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>36e517b8-47ca-4920-b242-d846caf9d0f4</v>
+      </c>
+      <c r="B66" t="str">
+        <v>LEMONNIER Thibault</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Chargé(e) d'Affaires</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Commercial Naskeo</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>6f10b670-44e5-4b45-8c4c-ff376a9ff2b5</v>
+      </c>
+      <c r="B67" t="str">
+        <v>LESIEUR Ewen</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Ingénieur(e) d'Etudes</v>
+      </c>
+      <c r="D67" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>e84b574b-7c90-482f-af56-ec92a661fefd</v>
+      </c>
+      <c r="B68" t="str">
+        <v>LHOTE Christophe</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Ingénieur(e) Mise en service</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Mise en service</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>dc1c5dde-7037-4896-ab0c-54c8a89d9616</v>
+      </c>
+      <c r="B69" t="str">
+        <v>LIMA Luisa</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Office Manager</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Office Management</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>741dc729-ab8f-4a4f-88f9-ffd78f3fc668</v>
+      </c>
+      <c r="B70" t="str">
+        <v>LUCAS Bruno</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Responsable Automaticien</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Automatisme</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>c6b73e90-5d53-4952-9626-60f679afd02c</v>
+      </c>
+      <c r="B71" t="str">
+        <v>LUGARDON Aurelien</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Président Directeur Général</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Direction Générale</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>d3c9044e-d501-4286-85ab-d15beeab40f6</v>
+      </c>
+      <c r="B72" t="str">
+        <v>MALIDOR Antoine</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Chargé(e) d'Affaires Nord-Ouest</v>
+      </c>
+      <c r="D72" t="str">
+        <v>Approvisionnement</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>02aa7530-1c27-4784-a1b3-dea15b453f40</v>
+      </c>
+      <c r="B73" t="str">
+        <v>MANGIN Diane</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Chargé(e) de Communication</v>
+      </c>
+      <c r="D73" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>dc333289-c5c3-4bac-9013-ca06cb135ea1</v>
+      </c>
+      <c r="B74" t="str">
+        <v>MANGIN Manon</v>
+      </c>
+      <c r="C74" t="str">
+        <v>Responsable Innovation, recherche et nouveaux métiers</v>
+      </c>
+      <c r="D74" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>a6c70c78-af73-4e57-a13d-3d36f0c98fe7</v>
+      </c>
+      <c r="B75" t="str">
+        <v>MARIE Aurélien</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Coordinateur(rice) Dessinateur-Projeteur</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Dessin</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>f9f02716-43ff-4b5a-b562-7e7d1b78779e</v>
+      </c>
+      <c r="B76" t="str">
+        <v>MARTIN Coline</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Responsable du Contrôle de gestion</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Contrôle de Gestion</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>17e506f2-8b1e-46e5-8641-84de7025c999</v>
+      </c>
+      <c r="B77" t="str">
+        <v>MARTIN SISTERON Florence</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Responsable Réglementaire</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Reglementation</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>149b85d9-3116-4c00-b5c2-fdf5af081e47</v>
+      </c>
+      <c r="B78" t="str">
+        <v>MEKDAD Safia</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Chargée des Ressources Humaines</v>
+      </c>
+      <c r="D78" t="str">
+        <v>Ressources Humaines</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>a44c6cd0-1ea5-4a9a-b6e2-dac49fcd7b06</v>
+      </c>
+      <c r="B79" t="str">
+        <v>MINARD Georges</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Responsable de Développement commercial</v>
+      </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>71c64620-fe4e-4ef0-b355-e52ecc3d6f69</v>
+      </c>
+      <c r="B80" t="str">
+        <v>MINGUET Corentin</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Chargé(e) d'Affaires</v>
+      </c>
+      <c r="D80" t="str">
+        <v>Commercial Naskeo</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>9144d1ff-71dd-4273-8b58-54927ad87773</v>
+      </c>
+      <c r="B81" t="str">
+        <v>MOLTO Hugues</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Chef de Projet Digital</v>
+      </c>
+      <c r="D81" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>4e4254bd-fd71-4933-a314-96826ce0a968</v>
+      </c>
+      <c r="B82" t="str">
+        <v>MORICEAU Guillaume</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Dessinateur(rice) Projeteur</v>
+      </c>
+      <c r="D82" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>c891a7d6-9b2e-400e-a039-ef5de4457f39</v>
+      </c>
+      <c r="B83" t="str">
+        <v>MOSER Louis</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Lead Recruiter</v>
+      </c>
+      <c r="D83" t="str">
+        <v>Ressources Humaines</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>497bf141-cdaf-4984-918d-8d86f8dbebf1</v>
+      </c>
+      <c r="B84" t="str">
+        <v>NAROLLES Nicolas</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Coordinateur(rice) Logistique</v>
+      </c>
+      <c r="D84" t="str">
+        <v>Logistique</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>20f86528-2731-410a-88b2-d5e096097840</v>
+      </c>
+      <c r="B85" t="str">
+        <v>NAUMANN Thorsten</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Country Manager</v>
+      </c>
+      <c r="D85" t="str">
+        <v>Montage de projet Int.</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>87360336-dc40-49ff-899c-729a1c5b4165</v>
+      </c>
+      <c r="B86" t="str">
+        <v>NGO Thao</v>
+      </c>
+      <c r="C86" t="str">
+        <v>Acheteur(se) Senior</v>
+      </c>
+      <c r="D86" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>7086c171-029a-4487-802d-60304c486a20</v>
+      </c>
+      <c r="B87" t="str">
+        <v>ORGET Claire</v>
+      </c>
+      <c r="C87" t="str">
+        <v>Responsable développement France</v>
+      </c>
+      <c r="D87" t="str">
+        <v>Montage de projet France</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>a89f8948-9761-4c64-ad27-f3da4bffc9d5</v>
+      </c>
+      <c r="B88" t="str">
+        <v>PAGEAUD Jules</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Business Developer</v>
+      </c>
+      <c r="D88" t="str">
+        <v>Business Developement</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>23c7a2c7-14aa-48cf-9dd0-c06c91f5c947</v>
+      </c>
+      <c r="B89" t="str">
+        <v>PAVAT Marion</v>
+      </c>
+      <c r="C89" t="str">
+        <v>Coordinateur(rice) Bureau d'Etudes</v>
+      </c>
+      <c r="D89" t="str">
+        <v>Bureau d'Etudes Naskeo</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>49d0e4b8-4c32-405f-8c9c-0c5a1fac334e</v>
+      </c>
+      <c r="B90" t="str">
+        <v>PERSAD SALAS Ranjit</v>
+      </c>
+      <c r="C90" t="str">
+        <v>Technicien(e) de Maintenance informatique et réseau</v>
+      </c>
+      <c r="D90" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>f87a4cdf-4e97-4037-ad82-e539160aff68</v>
+      </c>
+      <c r="B91" t="str">
+        <v>PICHON Charlotte</v>
+      </c>
+      <c r="C91" t="str">
+        <v>Experte agricole</v>
+      </c>
+      <c r="D91" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>811f2b1e-cecf-44af-8ee8-3b7c6927f898</v>
+      </c>
+      <c r="B92" t="str">
+        <v>POGUT Sébastien</v>
+      </c>
+      <c r="C92" t="str">
+        <v>Responsable de Site</v>
+      </c>
+      <c r="D92" t="str">
+        <v>Aunis Biogaz</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>908ff24d-16f1-4354-abc9-b5a9fa668b5d</v>
+      </c>
+      <c r="B93" t="str">
+        <v>RENNER Jérémy</v>
+      </c>
+      <c r="C93" t="str">
+        <v>Ingénieur(e) Maîtrise d'Oeuvre</v>
+      </c>
+      <c r="D93" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>409d2193-e1e4-46f7-95b5-3b1d23a58e16</v>
+      </c>
+      <c r="B94" t="str">
+        <v>REPPLINGER Mégane</v>
+      </c>
+      <c r="C94" t="str">
+        <v>Business Developer international Senior</v>
+      </c>
+      <c r="D94" t="str">
+        <v>Montage de projet Int.</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>da5059d2-6e95-4293-9895-20960de609c5</v>
+      </c>
+      <c r="B95" t="str">
+        <v>ROUGEBIEF Christelle</v>
+      </c>
+      <c r="C95" t="str">
+        <v>Président(e) Directeur(rice) Général(e)</v>
+      </c>
+      <c r="D95" t="str">
+        <v>Direction Générale</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>1041eae7-a58e-4c62-bd9b-3134f1e7eaf9</v>
+      </c>
+      <c r="B96" t="str">
+        <v>SAEZ Mélanie</v>
+      </c>
+      <c r="C96" t="str">
+        <v>Responsable Administratif et financier</v>
+      </c>
+      <c r="D96" t="str">
+        <v>Comptabilité</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>6858e0d4-d427-4af8-8d90-15f0ee5117d7</v>
+      </c>
+      <c r="B97" t="str">
+        <v>SARLOT Chloé</v>
+      </c>
+      <c r="C97" t="str">
+        <v>Chargé(e) de Communication</v>
+      </c>
+      <c r="D97" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>d4c90849-787b-4de3-8c05-79b28835fde2</v>
+      </c>
+      <c r="B98" t="str">
+        <v>SASSIAS Claire</v>
+      </c>
+      <c r="C98" t="str">
+        <v>Directeur(rice) Marketing et Communication</v>
+      </c>
+      <c r="D98" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>10ed374f-3bfd-45ef-b1bb-aa6d7c37e530</v>
+      </c>
+      <c r="B99" t="str">
+        <v>SIMERMAN Michel</v>
+      </c>
+      <c r="C99" t="str">
+        <v>Directeur(rice) d'exploitation</v>
+      </c>
+      <c r="D99" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>8bc56218-a294-42c4-82d8-ae220769e625</v>
+      </c>
+      <c r="B100" t="str">
+        <v>TIGNON Ludovic</v>
+      </c>
+      <c r="C100" t="str">
+        <v>Responsable Génie Civil</v>
+      </c>
+      <c r="D100" t="str">
+        <v>Génie Civil</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>542442c7-bb0b-4157-a34e-6a8053c05234</v>
+      </c>
+      <c r="B101" t="str">
+        <v>VERNEY Marie</v>
+      </c>
+      <c r="C101" t="str">
+        <v>Juriste</v>
+      </c>
+      <c r="D101" t="str">
+        <v>Juridique</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>46c195fd-a362-41fd-ba8a-53ba78e463e9</v>
+      </c>
+      <c r="B102" t="str">
+        <v>WILKS Jennifer</v>
+      </c>
+      <c r="C102" t="str">
+        <v>Office Manager</v>
+      </c>
+      <c r="D102" t="str">
+        <v>Office Management</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>603375ed-e3a2-49e0-a280-ae7cace0e67d</v>
+      </c>
+      <c r="B103" t="str">
+        <v>ZOWCZAK Martyna</v>
+      </c>
+      <c r="C103" t="str">
+        <v>Ingénieur(e) d'Etudes d'exploitation</v>
+      </c>
+      <c r="D103" t="str">
+        <v>Execution Naskeo</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D103"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B63"/>
+  <cols>
+    <col min="1" max="1" width="40.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>UUID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Département</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>50883e64-70f6-48e6-aa5e-0667eb533b4f</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Achats Keon</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>ab7d407b-18ff-4c82-b18b-915304577349</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Achats Naskeo</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>4e6afcea-c535-4abc-9c0e-a7834fc6832b</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Acquisitions</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>1a2c019a-1df5-44fd-a405-858494e9dfd2</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Approvisionnement</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>ea1ac616-3ea9-4084-8c4e-139f2234f3db</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Aunis Biogaz</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>98ea0187-3e70-4daf-9218-44d38aa77023</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Automatisme</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>c44ad9c3-a7ce-4ee3-a6e0-4f5bc79e5a4f</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Biogaz de Bel Air</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>ed779879-6522-46ea-b386-54c37313dffe</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Bureau d'Etudes Keon</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>107d6aa8-c362-4852-b7d4-24379abe74fb</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Bureau d'Etudes Naskeo</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>e8e81774-8a1c-479c-bf5d-8bfd99dd649e</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Business Developement</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>f47a9327-eed2-4cef-b436-b1c39c34d569</v>
+      </c>
+      <c r="B12" t="str">
+        <v>CERES</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>e0962c17-93df-4deb-8c69-7e9af25439e4</v>
+      </c>
+      <c r="B13" t="str">
+        <v>CERES Keon</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>90aa850e-83dc-44bc-a288-1f9679551982</v>
+      </c>
+      <c r="B14" t="str">
+        <v>CERES Sycomore</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>b834591a-fa5e-41fb-bf66-ff9231deac40</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Commercial Naskeo</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>fb4b9023-923a-4f58-993c-3a4e2002c502</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Commercial Sycomore</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>894745be-e528-4d7b-8483-7986d225f440</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Communication et Marketing</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>c1400dcd-52af-42db-8cdc-80e22173b076</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Comptabilité</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>05379788-9376-4a06-8241-b8e300f0842d</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Contrôle de Gestion</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>3439c517-1568-4533-9f3d-c634a30678c6</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Dessin</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>4a90eb54-f7c4-4b12-8996-d40097160df7</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Digital Keon</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>062a8478-48d9-4423-9a0c-98880ee7c65d</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Digital Sycomore</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>5f3a3959-7f47-4621-ad7c-e00e5f20f7fa</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Direction Administrative et Financière Keon</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>ca1b4a18-6866-46f1-9631-088b6e290300</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Direction Administrative et Financière Ter'Green</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>4aad1989-965f-46cc-bf06-8b6f611e5ea6</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Direction Commerciale</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>fbf34a95-4e6f-48b9-9548-a771cfb96133</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Direction du Développement</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>8d9edcc3-e7b2-46eb-82f4-f330c454fdc5</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Direction Générale</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>c5484372-a92d-448b-adf5-e84328aaca93</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Direction Operationelle Keon</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>d4938b99-4665-48a1-b1a2-e7e19f03e67c</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Direction Operationelle Sycomore</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>e3447836-7d65-4253-ac68-1df1ab2f9bf1</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Direction Travaux Keon</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>8f3669bb-7ecf-4536-b0d5-b6144a01ef8c</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Direction Travaux Naskeo</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>14f89310-e7f2-437a-97d7-5ce86e3a29c4</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Dole</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>6470a5c2-07cc-4a19-80e9-de78eb847559</v>
+      </c>
+      <c r="B33" t="str">
+        <v>E&amp;M</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>0448e1af-597f-4876-8772-837740aba3e7</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Execution Naskeo</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>87a44a36-520a-4df9-aa1f-4b8132887eea</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Exploitation Keon</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>3e8f9803-b497-4cf4-a433-4b41b256475a</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Exploitation Keon.bio</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>0a60cd94-7305-4eca-8868-a7ae953ec681</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Exploitation Sycomore</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>9be89016-e118-48cb-9f18-3170249e136d</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Exploitation Ter'Green</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>b09c8b28-a41b-443d-86fa-e27d0cd96c51</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Gatinais Déconditionnement</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>2cbafa44-019d-4e31-b447-61ddf11f3eb2</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Génie Civil</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>7736bc06-cc54-4e0c-8312-45ecdbae0136</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Juridique</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>2829a6b1-d9bd-47d8-90b2-3611b2f47f71</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Laboratoire</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>1e67a34c-4ecd-4ba8-baad-6c4a59fef2c4</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Les 3 dômes</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>39dc7015-8639-452b-84e4-b79b4f99bb39</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Logistique</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>a05eed86-79e5-48af-9644-097c29538981</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Maintenance</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>ecd5f64a-788f-42df-a5b2-2ae75fc96196</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Maîtrise d'ouvrage</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>371b43cb-9edd-45c8-8cf3-3f312e6c708f</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Mise en service</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>943690ab-3bc4-45ff-8ded-d1e176b23143</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Montage de projet France</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>9b7aa46f-e388-4293-a441-7ad256ea2e65</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Montage de projet Int.</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>68516016-e124-4923-ad30-f622137c805a</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Office Management</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>b2d4c485-f07f-4f5c-9159-defb61cbc275</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Partenariats Keon</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>2ab7c412-318f-4804-8e8b-cd03c33e54c2</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Partenariats Ter'Green</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>f4d78046-be7a-4886-bedd-7cfd0ee5716e</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Pole Exploitation Nord-Ouest</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>938bb36a-7719-4670-9ccb-abdccabb14f8</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Pole Exploitation Sud-Est Sycomore</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>541b2f7f-e138-4b71-95ee-2925e6894a31</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Pole Exploitation Sud-Est Ter'Green</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>c1fc2a56-9858-4706-b458-c5b10b12488c</v>
+      </c>
+      <c r="B56" t="str">
+        <v>R&amp;D Keon</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>94705b57-5c7c-4df5-8445-2852d042ec3b</v>
+      </c>
+      <c r="B57" t="str">
+        <v>R&amp;D Naskeo</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>6bbd0418-ca10-43a2-963b-a1573e76bece</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Réalisation</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>f4d32a6c-9f08-476b-9990-dcb6658a389d</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Reglementation</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>c66b703e-e3c9-4e12-84ef-20ee6ff157a6</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Ressources Humaines</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>aaf5581f-e88c-41a5-bc2c-2429e115f0d4</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Service IT/DIGITAL</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>bf2b99fc-eec9-44f2-9738-a5b23d9bee11</v>
+      </c>
+      <c r="B62" t="str">
+        <v>SG</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>9a9193ec-107b-4608-915a-40cfeb03391a</v>
+      </c>
+      <c r="B63" t="str">
+        <v>SPV</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B63"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B8"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="90.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Affectation type</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Description</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>fixed_user</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Personne fixée — colle son UUID dans « Affectation cible (UUID) »</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Rôle / job_title — colle l'UUID du job_title</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>manager_dispatch</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Un manager qui ré-affecte ensuite (cas BE) — UUID du manager</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>manager_requester</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Manager du demandeur (auto à la création) — UUID vide</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>requester</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Le demandeur lui-même — UUID vide</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>group</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Groupe d'utilisateurs — UUID du groupe</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>department</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Département cible — UUID du département</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I8"/>
   <cols>
     <col min="1" max="1" width="40.83203125" customWidth="1"/>
     <col min="2" max="2" width="42.83203125" customWidth="1"/>
@@ -1069,6 +3431,7 @@
     <col min="6" max="6" width="8.83203125" customWidth="1"/>
     <col min="7" max="7" width="14.83203125" customWidth="1"/>
     <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1096,6 +3459,9 @@
       <c r="H1" t="str">
         <v>État final</v>
       </c>
+      <c r="I1" t="str">
+        <v>Catégorie</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1122,6 +3488,9 @@
       <c r="H2" t="str">
         <v>non</v>
       </c>
+      <c r="I2" t="str">
+        <v>SOUMIS</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -1148,6 +3517,9 @@
       <c r="H3" t="str">
         <v>non</v>
       </c>
+      <c r="I3" t="str">
+        <v>EN_COURS</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -1174,6 +3546,9 @@
       <c r="H4" t="str">
         <v>non</v>
       </c>
+      <c r="I4" t="str">
+        <v>EN_ATTENTE_VALIDATION</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -1200,6 +3575,9 @@
       <c r="H5" t="str">
         <v>non</v>
       </c>
+      <c r="I5" t="str">
+        <v>EN_COURS</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -1226,6 +3604,9 @@
       <c r="H6" t="str">
         <v>oui</v>
       </c>
+      <c r="I6" t="str">
+        <v>TERMINE</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -1252,6 +3633,9 @@
       <c r="H7" t="str">
         <v>oui</v>
       </c>
+      <c r="I7" t="str">
+        <v>TERMINE</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -1278,19 +3662,22 @@
       <c r="H8" t="str">
         <v>oui</v>
       </c>
+      <c r="I8" t="str">
+        <v>TERMINE</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A37"/>
   <cols>
-    <col min="1" max="1" width="110.83203125" customWidth="1"/>
+    <col min="1" max="1" width="115.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1300,102 +3687,162 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>CE FICHIER contient 4 onglets :</v>
+        <v>ONGLETS :</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v xml:space="preserve">  1. SERVICE_ACHAT      : les 3 étapes existantes du flux Achat (à compléter avec États en sortie)</v>
+        <v xml:space="preserve">  1. SERVICE_ACHAT        — étapes existantes du flux Achat (à compléter)</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v xml:space="preserve">  2. NOUVELLES_ETAPES   : squelette pour saisir des étapes sur les flux IT/RH/Comm/Maintenance/Logistique/Innovation</v>
+        <v xml:space="preserve">  2. NOUVELLES_ETAPES     — saisie des étapes IT / RH / Comm / Maintenance / Logistique / Innovation</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v xml:space="preserve">  3. PROCESS_REFERENCE  : liste des ID des process pour recopier l'ID_processus dans NOUVELLES_ETAPES</v>
+        <v xml:space="preserve">  3. PROCESS_REFERENCE    — UUID des process à utiliser dans la colonne ID_processus</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v xml:space="preserve">  4. ETATS_PAR_FLUX     : liste des états par processus (duplique le bloc des 7 états par défaut pour chaque flux)</v>
+        <v xml:space="preserve">  4. PROFILES_REFERENCE   — UUID des utilisateurs (pour Affectation cible (UUID) quand type=fixed_user/manager_dispatch)</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v xml:space="preserve">  5. DEPARTMENTS_REFERENCE— UUID des départements (pour Affectation cible (UUID) quand type=department)</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>POUR SAISIR DES ÉTAPES SUR UN FLUX SANS ÉTAPES ACTUELLES (ex: IT - Demande d'intervention IT) :</v>
+        <v xml:space="preserve">  6. ASSIGNMENT_TYPES     — cheat-sheet des 7 modes d'affectation supportés</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v xml:space="preserve">  1. Va sur PROCESS_REFERENCE → copie l'ID_processus du flux concerné</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v xml:space="preserve">  2. Va sur NOUVELLES_ETAPES → colle l'ID dans ID_processus, remplis Processus, N°, Étape, Durée…</v>
+        <v xml:space="preserve">  7. ETATS_PAR_FLUX       — liste des états par processus + colonne Catégorie macro</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v xml:space="preserve">  3. Ajoute autant de lignes que d'étapes (la même ID_processus se répète)</v>
+        <v>⚠ AFFECTATION (nouveauté) :</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v xml:space="preserve">  L'affectation est définie au niveau du SOUS-PROCESSUS, pas de chaque étape.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>POUR DÉFINIR LES ÉTATS D'UN FLUX :</v>
+        <v xml:space="preserve">  → Remplis les colonnes « Affectation type » + « Affectation cible (UUID) » + « Affectation cible (nom) »</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v xml:space="preserve">  1. Va sur ETATS_PAR_FLUX</v>
+        <v xml:space="preserve">     UNIQUEMENT sur la 1ʳᵉ ligne (N°=1) de chaque ID_sous_processus.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v xml:space="preserve">  2. Pour chaque flux que tu veux configurer, recopie le bloc des 7 lignes (Code/Libellé/Couleur…) en renseignant</v>
+        <v xml:space="preserve">  → Pour les types « requester » et « manager_requester », laisse UUID vide.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v xml:space="preserve">     ID_processus + Processus correspondants. Modifie/ajoute/supprime selon besoin métier.</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>QUAND C'EST PRÊT :</v>
+        <v xml:space="preserve">  → Pour « fixed_user » / « manager_dispatch » : colle l'UUID depuis PROFILES_REFERENCE.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v xml:space="preserve">  → Pour « department » : colle l'UUID depuis DEPARTMENTS_REFERENCE.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v xml:space="preserve">  Renvoie ce fichier à Claude — il va :</v>
+        <v>POUR SAISIR DES ÉTAPES SUR UN FLUX SANS ÉTAPES (ex: IT - Demande d'intervention IT) :</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v xml:space="preserve">     • Mettre à jour les états en sortie pour SERVICE_ACHAT</v>
+        <v xml:space="preserve">  1. Va sur PROCESS_REFERENCE → copie l'ID_processus du flux concerné</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v xml:space="preserve">     • Créer les sub_process_templates + task_templates pour NOUVELLES_ETAPES (les flux qui n'avaient pas d'étapes)</v>
+        <v xml:space="preserve">  2. Va sur NOUVELLES_ETAPES → colle l'ID dans ID_processus + nom dans Processus</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v xml:space="preserve">     • Insérer les états dans request_states pour ETATS_PAR_FLUX</v>
+        <v xml:space="preserve">  3. Définis ID_sous_processus (UUID que tu inventes, format xxxxxxxx-xxxx-xxxx-xxxx-xxxxxxxxxxxx) +</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
+        <v xml:space="preserve">     Sous-processus (nom). Tu peux créer plusieurs sous-processus par flux.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v xml:space="preserve">  4. Pour chaque sous-processus, ajoute autant de lignes que d'étapes (N° 1, 2, 3…)</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v xml:space="preserve">  5. Sur la ligne N°=1 du sous-processus, renseigne les colonnes Affectation</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>POUR DÉFINIR LES ÉTATS D'UN FLUX :</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v xml:space="preserve">  → ETATS_PAR_FLUX : recopie le bloc des 7 lignes par flux, ajuste si besoin.</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v xml:space="preserve">  → Catégorie : SOUMIS | EN_COURS | EN_ATTENTE_VALIDATION | EN_ATTENTE_RETOUR_ADMIN | EN_ATTENTE_TRAVAUX | TERMINE</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>QUAND C'EST PRÊT :</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v xml:space="preserve">  Renvoie ce fichier à Claude — il génèrera :</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v xml:space="preserve">     • UPSERT sub_process_templates (assignment_type + target_*)</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v xml:space="preserve">     • INSERT task_templates (étapes + output_state_code)</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v xml:space="preserve">     • INSERT request_states (avec catégorie macro)</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
         <v xml:space="preserve">  Backup automatique avant écriture, comme pour le BE.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A37"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: régénère AUTRES_FLUX_parametrage.xlsx avec GROUPS_REFERENCE
</commit_message>
<xml_diff>
--- a/AUTRES_FLUX_parametrage.xlsx
+++ b/AUTRES_FLUX_parametrage.xlsx
@@ -8,9 +8,10 @@
     <sheet name="PROCESS_REFERENCE" sheetId="3" r:id="rId3"/>
     <sheet name="PROFILES_REFERENCE" sheetId="4" r:id="rId4"/>
     <sheet name="DEPARTMENTS_REFERENCE" sheetId="5" r:id="rId5"/>
-    <sheet name="ASSIGNMENT_TYPES" sheetId="6" r:id="rId6"/>
-    <sheet name="ETATS_PAR_FLUX" sheetId="7" r:id="rId7"/>
-    <sheet name="LISEZ-MOI" sheetId="8" r:id="rId8"/>
+    <sheet name="GROUPS_REFERENCE" sheetId="6" r:id="rId6"/>
+    <sheet name="ASSIGNMENT_TYPES" sheetId="7" r:id="rId7"/>
+    <sheet name="ETATS_PAR_FLUX" sheetId="8" r:id="rId8"/>
+    <sheet name="LISEZ-MOI" sheetId="9" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
@@ -3342,6 +3343,107 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D6"/>
+  <cols>
+    <col min="1" max="1" width="40.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="50.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>UUID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Groupe</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Description</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Membres</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>a2222222-2222-2222-2222-222222222222</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Comptabilité</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Groupe création fournisseur Divalto</v>
+      </c>
+      <c r="D2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>ed12ff20-0c81-48bb-adc4-402f4f5664c0</v>
+      </c>
+      <c r="B3" t="str">
+        <v>IT/DIGITAL</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>0f64dd74-463d-4ee0-8ada-53b840dbe886</v>
+      </c>
+      <c r="B4" t="str">
+        <v>RH</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>a1111111-1111-1111-1111-111111111111</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Service Achat</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Groupe vérifications fournisseurs</v>
+      </c>
+      <c r="D5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>43f37092-1366-4758-abbc-5b85fbcf355c</v>
+      </c>
+      <c r="B6" t="str">
+        <v>SERVICES GENERAUX</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B8"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
@@ -3419,7 +3521,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I8"/>
   <cols>
@@ -3673,9 +3775,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A37"/>
+  <dimension ref="A1:A39"/>
   <cols>
     <col min="1" max="1" width="115.83203125" customWidth="1"/>
   </cols>
@@ -3717,132 +3819,142 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v xml:space="preserve">  6. ASSIGNMENT_TYPES     — cheat-sheet des 7 modes d'affectation supportés</v>
+        <v xml:space="preserve">  6. GROUPS_REFERENCE     — UUID des groupes collaborateurs (pour Affectation cible (UUID) quand type=group)</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v xml:space="preserve">  7. ETATS_PAR_FLUX       — liste des états par processus + colonne Catégorie macro</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>⚠ AFFECTATION (nouveauté) :</v>
+        <v xml:space="preserve">  7. ASSIGNMENT_TYPES     — cheat-sheet des 7 modes d'affectation supportés</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v xml:space="preserve">  8. ETATS_PAR_FLUX       — liste des états par processus + colonne Catégorie macro</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v xml:space="preserve">  L'affectation est définie au niveau du SOUS-PROCESSUS, pas de chaque étape.</v>
+        <v>⚠ AFFECTATION (nouveauté) :</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v xml:space="preserve">  → Remplis les colonnes « Affectation type » + « Affectation cible (UUID) » + « Affectation cible (nom) »</v>
+        <v xml:space="preserve">  L'affectation est définie au niveau du SOUS-PROCESSUS, pas de chaque étape.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v xml:space="preserve">     UNIQUEMENT sur la 1ʳᵉ ligne (N°=1) de chaque ID_sous_processus.</v>
+        <v xml:space="preserve">  → Remplis les colonnes « Affectation type » + « Affectation cible (UUID) » + « Affectation cible (nom) »</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v xml:space="preserve">  → Pour les types « requester » et « manager_requester », laisse UUID vide.</v>
+        <v xml:space="preserve">     UNIQUEMENT sur la 1ʳᵉ ligne (N°=1) de chaque ID_sous_processus.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v xml:space="preserve">  → Pour « fixed_user » / « manager_dispatch » : colle l'UUID depuis PROFILES_REFERENCE.</v>
+        <v xml:space="preserve">  → Pour les types « requester » et « manager_requester », laisse UUID vide.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
+        <v xml:space="preserve">  → Pour « fixed_user » / « manager_dispatch » : colle l'UUID depuis PROFILES_REFERENCE.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
         <v xml:space="preserve">  → Pour « department » : colle l'UUID depuis DEPARTMENTS_REFERENCE.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>POUR SAISIR DES ÉTAPES SUR UN FLUX SANS ÉTAPES (ex: IT - Demande d'intervention IT) :</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v xml:space="preserve">  1. Va sur PROCESS_REFERENCE → copie l'ID_processus du flux concerné</v>
+        <v xml:space="preserve">  → Pour « group » : colle l'UUID depuis GROUPS_REFERENCE.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v xml:space="preserve">  2. Va sur NOUVELLES_ETAPES → colle l'ID dans ID_processus + nom dans Processus</v>
+        <v>POUR SAISIR DES ÉTAPES SUR UN FLUX SANS ÉTAPES (ex: IT - Demande d'intervention IT) :</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v xml:space="preserve">  3. Définis ID_sous_processus (UUID que tu inventes, format xxxxxxxx-xxxx-xxxx-xxxx-xxxxxxxxxxxx) +</v>
+        <v xml:space="preserve">  1. Va sur PROCESS_REFERENCE → copie l'ID_processus du flux concerné</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v xml:space="preserve">     Sous-processus (nom). Tu peux créer plusieurs sous-processus par flux.</v>
+        <v xml:space="preserve">  2. Va sur NOUVELLES_ETAPES → colle l'ID dans ID_processus + nom dans Processus</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v xml:space="preserve">  4. Pour chaque sous-processus, ajoute autant de lignes que d'étapes (N° 1, 2, 3…)</v>
+        <v xml:space="preserve">  3. Définis ID_sous_processus (UUID que tu inventes, format xxxxxxxx-xxxx-xxxx-xxxx-xxxxxxxxxxxx) +</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v xml:space="preserve">  5. Sur la ligne N°=1 du sous-processus, renseigne les colonnes Affectation</v>
+        <v xml:space="preserve">     Sous-processus (nom). Tu peux créer plusieurs sous-processus par flux.</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v xml:space="preserve">  4. Pour chaque sous-processus, ajoute autant de lignes que d'étapes (N° 1, 2, 3…)</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>POUR DÉFINIR LES ÉTATS D'UN FLUX :</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v xml:space="preserve">  → ETATS_PAR_FLUX : recopie le bloc des 7 lignes par flux, ajuste si besoin.</v>
+        <v xml:space="preserve">  5. Sur la ligne N°=1 du sous-processus, renseigne les colonnes Affectation</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v xml:space="preserve">  → Catégorie : SOUMIS | EN_COURS | EN_ATTENTE_VALIDATION | EN_ATTENTE_RETOUR_ADMIN | EN_ATTENTE_TRAVAUX | TERMINE</v>
+        <v>POUR DÉFINIR LES ÉTATS D'UN FLUX :</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v xml:space="preserve">  → ETATS_PAR_FLUX : recopie le bloc des 7 lignes par flux, ajuste si besoin.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>QUAND C'EST PRÊT :</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v xml:space="preserve">  Renvoie ce fichier à Claude — il génèrera :</v>
+        <v xml:space="preserve">  → Catégorie : SOUMIS | EN_COURS | EN_ATTENTE_VALIDATION | EN_ATTENTE_RETOUR_ADMIN | EN_ATTENTE_TRAVAUX | TERMINE</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v xml:space="preserve">     • UPSERT sub_process_templates (assignment_type + target_*)</v>
+        <v>QUAND C'EST PRÊT :</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v xml:space="preserve">     • INSERT task_templates (étapes + output_state_code)</v>
+        <v xml:space="preserve">  Renvoie ce fichier à Claude — il génèrera :</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v xml:space="preserve">     • INSERT request_states (avec catégorie macro)</v>
+        <v xml:space="preserve">     • UPSERT sub_process_templates (assignment_type + target_*)</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
+        <v xml:space="preserve">     • INSERT task_templates (étapes + output_state_code)</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v xml:space="preserve">     • INSERT request_states (avec catégorie macro)</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
         <v xml:space="preserve">  Backup automatique avant écriture, comme pour le BE.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A39"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(autres-flux): clarification affectation par étape (state-machine)
- LISEZ-MOI : distingue cas A (sous-processus → 1 affectataire, ligne N°=1
  uniquement) du cas B (chaque étape → affectataire différent, état-machine
  comme le flux nouveau fournisseur)
- SERVICE_ACHAT pré-rempli avec les vraies affectations actuellement actives
  via wf_workflows : Vérification → groupe Service Achat (a1111111),
  Création fournisseur → groupe Comptabilité (a2222222)

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AUTRES_FLUX_parametrage.xlsx
+++ b/AUTRES_FLUX_parametrage.xlsx
@@ -508,13 +508,13 @@
         <v>0</v>
       </c>
       <c r="J2" t="str">
-        <v>fixed_role</v>
+        <v>group</v>
       </c>
       <c r="K2" t="str">
-        <v/>
+        <v>a1111111-1111-1111-1111-111111111111</v>
       </c>
       <c r="L2" t="str">
-        <v/>
+        <v>Service Achat</v>
       </c>
       <c r="M2" t="str">
         <v>aucune</v>
@@ -529,7 +529,7 @@
         <v/>
       </c>
       <c r="Q2" t="str">
-        <v/>
+        <v>en_cours</v>
       </c>
     </row>
     <row r="3">
@@ -555,19 +555,19 @@
         <v>apres_precedente</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>1</v>
       </c>
       <c r="I3">
         <v>0</v>
       </c>
       <c r="J3" t="str">
-        <v/>
+        <v>group</v>
       </c>
       <c r="K3" t="str">
-        <v/>
+        <v>a2222222-2222-2222-2222-222222222222</v>
       </c>
       <c r="L3" t="str">
-        <v/>
+        <v>Comptabilité</v>
       </c>
       <c r="M3" t="str">
         <v>aucune</v>
@@ -582,7 +582,7 @@
         <v/>
       </c>
       <c r="Q3" t="str">
-        <v/>
+        <v>terminee</v>
       </c>
     </row>
     <row r="4">
@@ -614,13 +614,13 @@
         <v>0</v>
       </c>
       <c r="J4" t="str">
-        <v>fixed_user</v>
+        <v>group</v>
       </c>
       <c r="K4" t="str">
-        <v/>
+        <v>a1111111-1111-1111-1111-111111111111</v>
       </c>
       <c r="L4" t="str">
-        <v/>
+        <v>Service Achat</v>
       </c>
       <c r="M4" t="str">
         <v>aucune</v>
@@ -635,7 +635,7 @@
         <v/>
       </c>
       <c r="Q4" t="str">
-        <v/>
+        <v>terminee</v>
       </c>
     </row>
   </sheetData>
@@ -3777,7 +3777,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A39"/>
+  <dimension ref="A1:A47"/>
   <cols>
     <col min="1" max="1" width="115.83203125" customWidth="1"/>
   </cols>
@@ -3834,127 +3834,167 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>⚠ AFFECTATION (nouveauté) :</v>
+        <v>⚠ AFFECTATION — 2 cas à distinguer :</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v xml:space="preserve">  L'affectation est définie au niveau du SOUS-PROCESSUS, pas de chaque étape.</v>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v xml:space="preserve">  → Remplis les colonnes « Affectation type » + « Affectation cible (UUID) » + « Affectation cible (nom) »</v>
+        <v xml:space="preserve">  CAS A — toutes les étapes d'un sous-processus → MÊME affectataire :</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v xml:space="preserve">     UNIQUEMENT sur la 1ʳᵉ ligne (N°=1) de chaque ID_sous_processus.</v>
+        <v xml:space="preserve">     Remplis Affectation type/cible UNIQUEMENT sur la ligne N°=1.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v xml:space="preserve">  → Pour les types « requester » et « manager_requester », laisse UUID vide.</v>
+        <v xml:space="preserve">     → Je génère un sub_process_templates classique (affectation au niveau sous-processus).</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v xml:space="preserve">  → Pour « fixed_user » / « manager_dispatch » : colle l'UUID depuis PROFILES_REFERENCE.</v>
+        <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v xml:space="preserve">  → Pour « department » : colle l'UUID depuis DEPARTMENTS_REFERENCE.</v>
+        <v xml:space="preserve">  CAS B — chaque étape a un affectataire DIFFÉRENT (ex: Achat puis Comptabilité) :</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v xml:space="preserve">  → Pour « group » : colle l'UUID depuis GROUPS_REFERENCE.</v>
+        <v xml:space="preserve">     Remplis Affectation type/cible sur CHAQUE ligne (N°=1, 2, 3…).</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v xml:space="preserve">     → Je génère un workflow state-machine (wf_workflows/wf_steps), comme le flux</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>POUR SAISIR DES ÉTAPES SUR UN FLUX SANS ÉTAPES (ex: IT - Demande d'intervention IT) :</v>
+        <v xml:space="preserve">       « Demande de nouveau fournisseur » qui passe : Vérification (groupe Achat) →</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v xml:space="preserve">  1. Va sur PROCESS_REFERENCE → copie l'ID_processus du flux concerné</v>
+        <v xml:space="preserve">       Création (groupe Comptabilité) → Terminé.</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v xml:space="preserve">  2. Va sur NOUVELLES_ETAPES → colle l'ID dans ID_processus + nom dans Processus</v>
+        <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v xml:space="preserve">  3. Définis ID_sous_processus (UUID que tu inventes, format xxxxxxxx-xxxx-xxxx-xxxx-xxxxxxxxxxxx) +</v>
+        <v xml:space="preserve">  Pour les types « requester » et « manager_requester », laisse UUID vide.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v xml:space="preserve">     Sous-processus (nom). Tu peux créer plusieurs sous-processus par flux.</v>
+        <v xml:space="preserve">  Pour « fixed_user » / « manager_dispatch » : colle l'UUID depuis PROFILES_REFERENCE.</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v xml:space="preserve">  4. Pour chaque sous-processus, ajoute autant de lignes que d'étapes (N° 1, 2, 3…)</v>
+        <v xml:space="preserve">  Pour « department » : colle l'UUID depuis DEPARTMENTS_REFERENCE.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v xml:space="preserve">  5. Sur la ligne N°=1 du sous-processus, renseigne les colonnes Affectation</v>
+        <v xml:space="preserve">  Pour « group » : colle l'UUID depuis GROUPS_REFERENCE.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>POUR DÉFINIR LES ÉTATS D'UN FLUX :</v>
+        <v>POUR SAISIR DES ÉTAPES SUR UN FLUX SANS ÉTAPES (ex: IT - Demande d'intervention IT) :</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v xml:space="preserve">  → ETATS_PAR_FLUX : recopie le bloc des 7 lignes par flux, ajuste si besoin.</v>
+        <v xml:space="preserve">  1. Va sur PROCESS_REFERENCE → copie l'ID_processus du flux concerné</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v xml:space="preserve">  → Catégorie : SOUMIS | EN_COURS | EN_ATTENTE_VALIDATION | EN_ATTENTE_RETOUR_ADMIN | EN_ATTENTE_TRAVAUX | TERMINE</v>
+        <v xml:space="preserve">  2. Va sur NOUVELLES_ETAPES → colle l'ID dans ID_processus + nom dans Processus</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v xml:space="preserve">  3. Définis ID_sous_processus (UUID que tu inventes, format xxxxxxxx-xxxx-xxxx-xxxx-xxxxxxxxxxxx) +</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>QUAND C'EST PRÊT :</v>
+        <v xml:space="preserve">     Sous-processus (nom). Tu peux créer plusieurs sous-processus par flux.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v xml:space="preserve">  Renvoie ce fichier à Claude — il génèrera :</v>
+        <v xml:space="preserve">  4. Pour chaque sous-processus, ajoute autant de lignes que d'étapes (N° 1, 2, 3…)</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v xml:space="preserve">     • UPSERT sub_process_templates (assignment_type + target_*)</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v xml:space="preserve">     • INSERT task_templates (étapes + output_state_code)</v>
+        <v xml:space="preserve">  5. Sur la ligne N°=1 du sous-processus, renseigne les colonnes Affectation</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v xml:space="preserve">     • INSERT request_states (avec catégorie macro)</v>
+        <v>POUR DÉFINIR LES ÉTATS D'UN FLUX :</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
+        <v xml:space="preserve">  → ETATS_PAR_FLUX : recopie le bloc des 7 lignes par flux, ajuste si besoin.</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v xml:space="preserve">  → Catégorie : SOUMIS | EN_COURS | EN_ATTENTE_VALIDATION | EN_ATTENTE_RETOUR_ADMIN | EN_ATTENTE_TRAVAUX | TERMINE</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>QUAND C'EST PRÊT :</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v xml:space="preserve">  Renvoie ce fichier à Claude — il génèrera :</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v xml:space="preserve">     • UPSERT sub_process_templates (assignment_type + target_*)</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v xml:space="preserve">     • INSERT task_templates (étapes + output_state_code)</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v xml:space="preserve">     • INSERT request_states (avec catégorie macro)</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
         <v xml:space="preserve">  Backup automatique avant écriture, comme pour le BE.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A39"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A47"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(autres-flux): onglets EXISTANT + TABLE_EFFECTS
- Nouveau snapshot _flows-snapshot.json : dump complet des process configurés
  en DB hors BE (32 lignes process/sp/tt — Comptabilité, Gestion régl., Innovation,
  Onboarding, QSE, Service Achat, Service Maintenance, Service Marketing, Support
  IT/DIGITAL avec ses 6 sous-processus)
- Onglet EXISTANT (read-only) : visualisation de toutes les configurations
  actuelles (affectation au niveau sous-processus + override target_group_id
  au niveau étape)
- Onglet TABLE_EFFECTS : documentation des effets de bord sur les tables
  métier (supplier_waiting_approval → suppliers, nc_declarations / nc_actions,
  inno_demandes, demande_materiel)
- LISEZ-MOI mis à jour avec les 2 nouveaux onglets en tête

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AUTRES_FLUX_parametrage.xlsx
+++ b/AUTRES_FLUX_parametrage.xlsx
@@ -3,15 +3,17 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="SERVICE_ACHAT" sheetId="1" r:id="rId1"/>
-    <sheet name="NOUVELLES_ETAPES" sheetId="2" r:id="rId2"/>
-    <sheet name="PROCESS_REFERENCE" sheetId="3" r:id="rId3"/>
-    <sheet name="PROFILES_REFERENCE" sheetId="4" r:id="rId4"/>
-    <sheet name="DEPARTMENTS_REFERENCE" sheetId="5" r:id="rId5"/>
-    <sheet name="GROUPS_REFERENCE" sheetId="6" r:id="rId6"/>
-    <sheet name="ASSIGNMENT_TYPES" sheetId="7" r:id="rId7"/>
-    <sheet name="ETATS_PAR_FLUX" sheetId="8" r:id="rId8"/>
-    <sheet name="LISEZ-MOI" sheetId="9" r:id="rId9"/>
+    <sheet name="EXISTANT" sheetId="1" r:id="rId1"/>
+    <sheet name="TABLE_EFFECTS" sheetId="2" r:id="rId2"/>
+    <sheet name="SERVICE_ACHAT" sheetId="3" r:id="rId3"/>
+    <sheet name="NOUVELLES_ETAPES" sheetId="4" r:id="rId4"/>
+    <sheet name="PROCESS_REFERENCE" sheetId="5" r:id="rId5"/>
+    <sheet name="PROFILES_REFERENCE" sheetId="6" r:id="rId6"/>
+    <sheet name="DEPARTMENTS_REFERENCE" sheetId="7" r:id="rId7"/>
+    <sheet name="GROUPS_REFERENCE" sheetId="8" r:id="rId8"/>
+    <sheet name="ASSIGNMENT_TYPES" sheetId="9" r:id="rId9"/>
+    <sheet name="ETATS_PAR_FLUX" sheetId="10" r:id="rId10"/>
+    <sheet name="LISEZ-MOI" sheetId="11" r:id="rId11"/>
   </sheets>
 </workbook>
 </file>
@@ -405,6 +407,2988 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Q40"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="42.83203125" customWidth="1"/>
+    <col min="3" max="3" width="6.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="32.83203125" customWidth="1"/>
+    <col min="6" max="6" width="38.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="6.83203125" customWidth="1"/>
+    <col min="9" max="9" width="48.83203125" customWidth="1"/>
+    <col min="10" max="10" width="8.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.83203125" customWidth="1"/>
+    <col min="12" max="12" width="22.83203125" customWidth="1"/>
+    <col min="13" max="13" width="38.83203125" customWidth="1"/>
+    <col min="14" max="14" width="12.83203125" customWidth="1"/>
+    <col min="15" max="15" width="38.83203125" customWidth="1"/>
+    <col min="16" max="16" width="38.83203125" customWidth="1"/>
+    <col min="17" max="17" width="38.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Processus</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Sous-processus</v>
+      </c>
+      <c r="C1" t="str">
+        <v>N° sp</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Affectation type (sp)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Affectation cible (sp)</v>
+      </c>
+      <c r="F1" t="str">
+        <v>UUID cible (sp)</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Type cible</v>
+      </c>
+      <c r="H1" t="str">
+        <v>N° étape</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Étape</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Durée (j)</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Démarrage</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Override groupe (étape)</v>
+      </c>
+      <c r="M1" t="str">
+        <v>UUID override (étape)</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Validation</v>
+      </c>
+      <c r="O1" t="str">
+        <v>ID processus</v>
+      </c>
+      <c r="P1" t="str">
+        <v>ID sous-processus</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>ID étape</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>COMPTABILITÉ</v>
+      </c>
+      <c r="B2" t="str">
+        <v>AJOUT DE CLIENT</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2" t="str">
+        <v>manager_dispatch</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Comptabilité</v>
+      </c>
+      <c r="F2" t="str">
+        <v>c1400dcd-52af-42db-8cdc-80e22173b076</v>
+      </c>
+      <c r="G2" t="str">
+        <v>department</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2" t="str">
+        <v>CREATION CLIENT</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v>none</v>
+      </c>
+      <c r="O2" t="str">
+        <v>2267fe2c-8ced-406b-969b-a21dadc30189</v>
+      </c>
+      <c r="P2" t="str">
+        <v>b9eb6f86-e4d5-4c73-9776-24f8f8c2ad3e</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>30714907-a3ae-4fdf-a89c-c3cbd763499f</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>GESTION REGLEMENTAIRE SITE EN EXPLOITATION</v>
+      </c>
+      <c r="B3" t="str">
+        <v>RAPPORT ANNUEL ICPE</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3" t="str">
+        <v>manager_dispatch</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Exploitation Keon.bio</v>
+      </c>
+      <c r="F3" t="str">
+        <v>3e8f9803-b497-4cf4-a433-4b41b256475a</v>
+      </c>
+      <c r="G3" t="str">
+        <v>department</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3" t="str">
+        <v>REDIGER V0 - RAPPORT ANNUEL ICPE</v>
+      </c>
+      <c r="J3">
+        <v>7</v>
+      </c>
+      <c r="K3" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v>none</v>
+      </c>
+      <c r="O3" t="str">
+        <v>349182ad-008a-4304-9297-33855bc2baac</v>
+      </c>
+      <c r="P3" t="str">
+        <v>d8603c71-e82f-4317-b6f6-5d403742cf1c</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>a64ada5b-3a37-4efa-a5aa-dfa97d3c565e</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>GESTION REGLEMENTAIRE SITE EN EXPLOITATION</v>
+      </c>
+      <c r="B4" t="str">
+        <v>RAPPORT ANNUEL ICPE</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4" t="str">
+        <v>manager_dispatch</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Exploitation Keon.bio</v>
+      </c>
+      <c r="F4" t="str">
+        <v>3e8f9803-b497-4cf4-a433-4b41b256475a</v>
+      </c>
+      <c r="G4" t="str">
+        <v>department</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4" t="str">
+        <v>RECUPERER DONNES ANNUELLE DE PROD - RAPPORT ANNUEL ICPE</v>
+      </c>
+      <c r="J4">
+        <v>7</v>
+      </c>
+      <c r="K4" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v>none</v>
+      </c>
+      <c r="O4" t="str">
+        <v>349182ad-008a-4304-9297-33855bc2baac</v>
+      </c>
+      <c r="P4" t="str">
+        <v>d8603c71-e82f-4317-b6f6-5d403742cf1c</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>9f05938e-bbb8-4d4d-bfa9-afdff02d0935</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>GESTION REGLEMENTAIRE SITE EN EXPLOITATION</v>
+      </c>
+      <c r="B5" t="str">
+        <v>RAPPORT RED3</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="str">
+        <v>manager_dispatch</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+      <c r="I5" t="str">
+        <v>(aucune tâche-template)</v>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v>349182ad-008a-4304-9297-33855bc2baac</v>
+      </c>
+      <c r="P5" t="str">
+        <v>fbe38955-b6e8-4b23-8e52-1dc48ec0d92b</v>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Innovation</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Demande Innovation</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6" t="str">
+        <v>fixed_user</v>
+      </c>
+      <c r="E6" t="str">
+        <v>MANGIN Manon</v>
+      </c>
+      <c r="F6" t="str">
+        <v>dc333289-c5c3-4bac-9013-ca06cb135ea1</v>
+      </c>
+      <c r="G6" t="str">
+        <v>user</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Instruire la demande</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v>none</v>
+      </c>
+      <c r="O6" t="str">
+        <v>a1b2c3d4-0000-4000-a000-000000000001</v>
+      </c>
+      <c r="P6" t="str">
+        <v>b2c3d4e5-0000-4000-b000-000000000001</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>99493a04-b371-432f-b5e7-702634825e50</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Innovation</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Demande Innovation</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7" t="str">
+        <v>fixed_user</v>
+      </c>
+      <c r="E7" t="str">
+        <v>MANGIN Manon</v>
+      </c>
+      <c r="F7" t="str">
+        <v>dc333289-c5c3-4bac-9013-ca06cb135ea1</v>
+      </c>
+      <c r="G7" t="str">
+        <v>user</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Présenter au CODIR</v>
+      </c>
+      <c r="J7">
+        <v>1</v>
+      </c>
+      <c r="K7" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v>none</v>
+      </c>
+      <c r="O7" t="str">
+        <v>a1b2c3d4-0000-4000-a000-000000000001</v>
+      </c>
+      <c r="P7" t="str">
+        <v>b2c3d4e5-0000-4000-b000-000000000001</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>9b1bffb0-f1de-471c-8bc8-34c395d13f82</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Innovation</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Demande Innovation</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8" t="str">
+        <v>fixed_user</v>
+      </c>
+      <c r="E8" t="str">
+        <v>MANGIN Manon</v>
+      </c>
+      <c r="F8" t="str">
+        <v>dc333289-c5c3-4bac-9013-ca06cb135ea1</v>
+      </c>
+      <c r="G8" t="str">
+        <v>user</v>
+      </c>
+      <c r="H8">
+        <v>2</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Mettre en oeuvre le projet</v>
+      </c>
+      <c r="J8">
+        <v>10</v>
+      </c>
+      <c r="K8" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v>none</v>
+      </c>
+      <c r="O8" t="str">
+        <v>a1b2c3d4-0000-4000-a000-000000000001</v>
+      </c>
+      <c r="P8" t="str">
+        <v>b2c3d4e5-0000-4000-b000-000000000001</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>3abf2f42-543d-48cd-a28b-f6d0f2764267</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>ONBOARDING</v>
+      </c>
+      <c r="B9" t="str">
+        <v>ONBOARDING</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="E9" t="str">
+        <v>TECHNICIEN IT</v>
+      </c>
+      <c r="F9" t="str">
+        <v>640b7ff1-df57-4bab-a287-67f04a3c4f1e</v>
+      </c>
+      <c r="G9" t="str">
+        <v>job_title</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9" t="str">
+        <v>PREPARER LE POSTE DE TRAVAIL - ONBOARDING-IT</v>
+      </c>
+      <c r="J9">
+        <v>10</v>
+      </c>
+      <c r="K9" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v>none</v>
+      </c>
+      <c r="O9" t="str">
+        <v>128268b0-e9d0-42b2-bc98-8de667671f9c</v>
+      </c>
+      <c r="P9" t="str">
+        <v>01f4023b-9cd8-45ef-8e38-c7d37246047f</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>9c1f22c5-2372-4c45-9e00-562c48e0d075</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>ONBOARDING</v>
+      </c>
+      <c r="B10" t="str">
+        <v>MUTATION</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Preparation outils de travail</v>
+      </c>
+      <c r="J10">
+        <v>1</v>
+      </c>
+      <c r="K10" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v>none</v>
+      </c>
+      <c r="O10" t="str">
+        <v>128268b0-e9d0-42b2-bc98-8de667671f9c</v>
+      </c>
+      <c r="P10" t="str">
+        <v>4442cbf4-71f5-487b-8319-140aa121d7bc</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>9309450c-4bcd-4737-93f6-863136da5500</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>ONBOARDING</v>
+      </c>
+      <c r="B11" t="str">
+        <v>OFFBOARDING</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+      <c r="D11" t="str">
+        <v>fixed_user</v>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+      <c r="I11" t="str">
+        <v>(aucune tâche-template)</v>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v/>
+      </c>
+      <c r="O11" t="str">
+        <v>128268b0-e9d0-42b2-bc98-8de667671f9c</v>
+      </c>
+      <c r="P11" t="str">
+        <v>9a190d0c-33a2-4e51-a0ea-987fac4e07ad</v>
+      </c>
+      <c r="Q11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>ONBOARDING</v>
+      </c>
+      <c r="B12" t="str">
+        <v>PROMOTION</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="D12" t="str">
+        <v>fixed_user</v>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+      <c r="I12" t="str">
+        <v>(aucune tâche-template)</v>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
+      <c r="M12" t="str">
+        <v/>
+      </c>
+      <c r="N12" t="str">
+        <v/>
+      </c>
+      <c r="O12" t="str">
+        <v>128268b0-e9d0-42b2-bc98-8de667671f9c</v>
+      </c>
+      <c r="P12" t="str">
+        <v>62c29879-4c08-4b82-adbb-d9edcbd56ccf</v>
+      </c>
+      <c r="Q12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>QUALITÉ SECURITE ENVIRONNEMENT</v>
+      </c>
+      <c r="B13" t="str">
+        <v>DECLARATION DE NON CONFORMITE</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13" t="str">
+        <v>fixed_user</v>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+      <c r="I13" t="str">
+        <v>(aucune tâche-template — workflow géré via nc_declarations)</v>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
+        <v/>
+      </c>
+      <c r="M13" t="str">
+        <v/>
+      </c>
+      <c r="N13" t="str">
+        <v/>
+      </c>
+      <c r="O13" t="str">
+        <v>697fdfee-7a64-4193-af2f-bece2da44d8e</v>
+      </c>
+      <c r="P13" t="str">
+        <v>82f8552e-e09c-45d1-a4f7-45a572138ee3</v>
+      </c>
+      <c r="Q13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>SERVICE ACHAT</v>
+      </c>
+      <c r="B14" t="str">
+        <v>DEMANDE DE NOUVEAU FOURNISSEUR</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="E14" t="str">
+        <v>(via task_templates.target_group_id)</v>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v>per_task_override</v>
+      </c>
+      <c r="H14">
+        <v>1</v>
+      </c>
+      <c r="I14" t="str">
+        <v>Vérification fournisseur</v>
+      </c>
+      <c r="J14">
+        <v>1</v>
+      </c>
+      <c r="K14" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Service Achat</v>
+      </c>
+      <c r="M14" t="str">
+        <v>a1111111-1111-1111-1111-111111111111</v>
+      </c>
+      <c r="N14" t="str">
+        <v>none</v>
+      </c>
+      <c r="O14" t="str">
+        <v>b1111111-1111-1111-1111-111111111111</v>
+      </c>
+      <c r="P14" t="str">
+        <v>c1111111-1111-1111-1111-111111111111</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>d1111111-1111-1111-1111-111111111111</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>SERVICE ACHAT</v>
+      </c>
+      <c r="B15" t="str">
+        <v>DEMANDE DE NOUVEAU FOURNISSEUR</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="E15" t="str">
+        <v>(via task_templates.target_group_id)</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v>per_task_override</v>
+      </c>
+      <c r="H15">
+        <v>2</v>
+      </c>
+      <c r="I15" t="str">
+        <v>Création fournisseur</v>
+      </c>
+      <c r="J15">
+        <v>1</v>
+      </c>
+      <c r="K15" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L15" t="str">
+        <v>Comptabilité</v>
+      </c>
+      <c r="M15" t="str">
+        <v>a2222222-2222-2222-2222-222222222222</v>
+      </c>
+      <c r="N15" t="str">
+        <v>none</v>
+      </c>
+      <c r="O15" t="str">
+        <v>b1111111-1111-1111-1111-111111111111</v>
+      </c>
+      <c r="P15" t="str">
+        <v>c1111111-1111-1111-1111-111111111111</v>
+      </c>
+      <c r="Q15" t="str">
+        <v>d2222222-2222-2222-2222-222222222222</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>SERVICE ACHAT</v>
+      </c>
+      <c r="B16" t="str">
+        <v>DEMANDE DIVERSES SERVICE ACHAT (HORS NOUVEAU FOURNISSEUR)</v>
+      </c>
+      <c r="C16">
+        <v>2</v>
+      </c>
+      <c r="D16" t="str">
+        <v>fixed_user</v>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16" t="str">
+        <v>REPONDRE AU TICKET</v>
+      </c>
+      <c r="J16">
+        <v>1</v>
+      </c>
+      <c r="K16" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L16" t="str">
+        <v/>
+      </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
+        <v>none</v>
+      </c>
+      <c r="O16" t="str">
+        <v>b1111111-1111-1111-1111-111111111111</v>
+      </c>
+      <c r="P16" t="str">
+        <v>951d6c3c-82ca-4468-97ca-ca51275da573</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>35a65b15-63ae-4d31-94dc-f0f18d39339c</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>SERVICE MAINTENANCE</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Demande de matériel</v>
+      </c>
+      <c r="C17">
+        <v>0</v>
+      </c>
+      <c r="D17" t="str">
+        <v>fixed_user</v>
+      </c>
+      <c r="E17" t="str">
+        <v>BERTRAND Valentin</v>
+      </c>
+      <c r="F17" t="str">
+        <v>81750c79-efb6-48e2-8788-0ec9a6f13b68</v>
+      </c>
+      <c r="G17" t="str">
+        <v>user</v>
+      </c>
+      <c r="H17">
+        <v>0</v>
+      </c>
+      <c r="I17" t="str">
+        <v>{sous_processus} - Traitement commande maintenance</v>
+      </c>
+      <c r="J17">
+        <v>10</v>
+      </c>
+      <c r="K17" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
+      <c r="M17" t="str">
+        <v/>
+      </c>
+      <c r="N17" t="str">
+        <v>none</v>
+      </c>
+      <c r="O17" t="str">
+        <v>a1b2c3d4-e5f6-7890-abcd-ef1234567890</v>
+      </c>
+      <c r="P17" t="str">
+        <v>b2c3d4e5-f6a7-8901-bcde-f12345678901</v>
+      </c>
+      <c r="Q17" t="str">
+        <v>9caaf507-2b1a-49b4-9190-c2d841da9497</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>SERVICE MARKETING</v>
+      </c>
+      <c r="B18" t="str">
+        <v>RESERVATION DES STANDS POUR LES SALONS</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18" t="str">
+        <v>manager_dispatch</v>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18">
+        <v>1</v>
+      </c>
+      <c r="I18" t="str">
+        <v>RESERVER SALON</v>
+      </c>
+      <c r="J18">
+        <v>5</v>
+      </c>
+      <c r="K18" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
+      <c r="M18" t="str">
+        <v/>
+      </c>
+      <c r="N18" t="str">
+        <v>none</v>
+      </c>
+      <c r="O18" t="str">
+        <v>a87c0649-2a71-471e-95e4-7e0ae68f5cf8</v>
+      </c>
+      <c r="P18" t="str">
+        <v>1cf20f9f-b82b-4f07-8d98-8b87218cad21</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>7fc87c10-b865-47fc-85b7-3ccfab08bd72</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>SERVICE MARKETING</v>
+      </c>
+      <c r="B19" t="str">
+        <v>RESERVATION DES STANDS POUR LES SALONS</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19" t="str">
+        <v>manager_dispatch</v>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19">
+        <v>2</v>
+      </c>
+      <c r="I19" t="str">
+        <v>ORGANISER TRANSPORT</v>
+      </c>
+      <c r="J19">
+        <v>3</v>
+      </c>
+      <c r="K19" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L19" t="str">
+        <v/>
+      </c>
+      <c r="M19" t="str">
+        <v/>
+      </c>
+      <c r="N19" t="str">
+        <v>none</v>
+      </c>
+      <c r="O19" t="str">
+        <v>a87c0649-2a71-471e-95e4-7e0ae68f5cf8</v>
+      </c>
+      <c r="P19" t="str">
+        <v>1cf20f9f-b82b-4f07-8d98-8b87218cad21</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>904aaefc-47e8-4a88-a97d-3896cb943594</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B20" t="str">
+        <v>OUVERTURE DOSSIER SHAREPOINT</v>
+      </c>
+      <c r="C20">
+        <v>2</v>
+      </c>
+      <c r="D20" t="str">
+        <v>fixed_user</v>
+      </c>
+      <c r="E20" t="str">
+        <v>PERSAD SALAS Ranjit</v>
+      </c>
+      <c r="F20" t="str">
+        <v>49d0e4b8-4c32-405f-8c9c-0c5a1fac334e</v>
+      </c>
+      <c r="G20" t="str">
+        <v>user</v>
+      </c>
+      <c r="H20">
+        <v>1</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Création de la structure</v>
+      </c>
+      <c r="J20">
+        <v>1</v>
+      </c>
+      <c r="K20" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L20" t="str">
+        <v/>
+      </c>
+      <c r="M20" t="str">
+        <v/>
+      </c>
+      <c r="N20" t="str">
+        <v>none</v>
+      </c>
+      <c r="O20" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P20" t="str">
+        <v>22222222-2222-2222-2222-222222222222</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>06e3b523-bcd0-40cc-b563-6fe59b712d9f</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B21" t="str">
+        <v>OUVERTURE DOSSIER SHAREPOINT</v>
+      </c>
+      <c r="C21">
+        <v>2</v>
+      </c>
+      <c r="D21" t="str">
+        <v>fixed_user</v>
+      </c>
+      <c r="E21" t="str">
+        <v>PERSAD SALAS Ranjit</v>
+      </c>
+      <c r="F21" t="str">
+        <v>49d0e4b8-4c32-405f-8c9c-0c5a1fac334e</v>
+      </c>
+      <c r="G21" t="str">
+        <v>user</v>
+      </c>
+      <c r="H21">
+        <v>2</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Configuration des permissions</v>
+      </c>
+      <c r="J21">
+        <v>1</v>
+      </c>
+      <c r="K21" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+      <c r="M21" t="str">
+        <v/>
+      </c>
+      <c r="N21" t="str">
+        <v>none</v>
+      </c>
+      <c r="O21" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P21" t="str">
+        <v>22222222-2222-2222-2222-222222222222</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>27f0aedd-7072-43c2-8d08-b9b03bb8825f</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B22" t="str">
+        <v>OUVERTURE DOSSIER SHAREPOINT</v>
+      </c>
+      <c r="C22">
+        <v>2</v>
+      </c>
+      <c r="D22" t="str">
+        <v>fixed_user</v>
+      </c>
+      <c r="E22" t="str">
+        <v>PERSAD SALAS Ranjit</v>
+      </c>
+      <c r="F22" t="str">
+        <v>49d0e4b8-4c32-405f-8c9c-0c5a1fac334e</v>
+      </c>
+      <c r="G22" t="str">
+        <v>user</v>
+      </c>
+      <c r="H22">
+        <v>3</v>
+      </c>
+      <c r="I22" t="str">
+        <v>Notification aux utilisateurs</v>
+      </c>
+      <c r="J22">
+        <v>1</v>
+      </c>
+      <c r="K22" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L22" t="str">
+        <v/>
+      </c>
+      <c r="M22" t="str">
+        <v/>
+      </c>
+      <c r="N22" t="str">
+        <v>none</v>
+      </c>
+      <c r="O22" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P22" t="str">
+        <v>22222222-2222-2222-2222-222222222222</v>
+      </c>
+      <c r="Q22" t="str">
+        <v>b5561df0-e91f-43bd-a102-74afe2d78d48</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B23" t="str">
+        <v>SUPPORT DIVALTO</v>
+      </c>
+      <c r="C23">
+        <v>3</v>
+      </c>
+      <c r="D23" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="E23" t="str">
+        <v>CHEF DE PROJET DIGITAL</v>
+      </c>
+      <c r="F23" t="str">
+        <v>59297fc0-b709-4908-bdfe-be7c04c0eb46</v>
+      </c>
+      <c r="G23" t="str">
+        <v>job_title</v>
+      </c>
+      <c r="H23">
+        <v>1</v>
+      </c>
+      <c r="I23" t="str">
+        <v>Analyse de la demande</v>
+      </c>
+      <c r="J23">
+        <v>1</v>
+      </c>
+      <c r="K23" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L23" t="str">
+        <v/>
+      </c>
+      <c r="M23" t="str">
+        <v/>
+      </c>
+      <c r="N23" t="str">
+        <v>none</v>
+      </c>
+      <c r="O23" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P23" t="str">
+        <v>33333333-3333-3333-3333-333333333333</v>
+      </c>
+      <c r="Q23" t="str">
+        <v>30a16734-fc45-4c23-ace5-3247f5bfb10f</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B24" t="str">
+        <v>SUPPORT DIVALTO</v>
+      </c>
+      <c r="C24">
+        <v>3</v>
+      </c>
+      <c r="D24" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="E24" t="str">
+        <v>CHEF DE PROJET DIGITAL</v>
+      </c>
+      <c r="F24" t="str">
+        <v>59297fc0-b709-4908-bdfe-be7c04c0eb46</v>
+      </c>
+      <c r="G24" t="str">
+        <v>job_title</v>
+      </c>
+      <c r="H24">
+        <v>2</v>
+      </c>
+      <c r="I24" t="str">
+        <v>Intervention sur Divalto</v>
+      </c>
+      <c r="J24">
+        <v>3</v>
+      </c>
+      <c r="K24" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L24" t="str">
+        <v/>
+      </c>
+      <c r="M24" t="str">
+        <v/>
+      </c>
+      <c r="N24" t="str">
+        <v>none</v>
+      </c>
+      <c r="O24" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P24" t="str">
+        <v>33333333-3333-3333-3333-333333333333</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>5dedcc2a-c42d-40d3-890e-f611312346b5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B25" t="str">
+        <v>SUPPORT DIVALTO</v>
+      </c>
+      <c r="C25">
+        <v>3</v>
+      </c>
+      <c r="D25" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="E25" t="str">
+        <v>CHEF DE PROJET DIGITAL</v>
+      </c>
+      <c r="F25" t="str">
+        <v>59297fc0-b709-4908-bdfe-be7c04c0eb46</v>
+      </c>
+      <c r="G25" t="str">
+        <v>job_title</v>
+      </c>
+      <c r="H25">
+        <v>3</v>
+      </c>
+      <c r="I25" t="str">
+        <v>Tests et validation métier</v>
+      </c>
+      <c r="J25">
+        <v>2</v>
+      </c>
+      <c r="K25" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L25" t="str">
+        <v/>
+      </c>
+      <c r="M25" t="str">
+        <v/>
+      </c>
+      <c r="N25" t="str">
+        <v>none</v>
+      </c>
+      <c r="O25" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P25" t="str">
+        <v>33333333-3333-3333-3333-333333333333</v>
+      </c>
+      <c r="Q25" t="str">
+        <v>d40c07e7-b337-49d7-935b-4068ef91b035</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B26" t="str">
+        <v>SUPPORT PIPEDRIVE</v>
+      </c>
+      <c r="C26">
+        <v>4</v>
+      </c>
+      <c r="D26" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="E26" t="str">
+        <v>CHEF DE PROJET DIGITAL</v>
+      </c>
+      <c r="F26" t="str">
+        <v>59297fc0-b709-4908-bdfe-be7c04c0eb46</v>
+      </c>
+      <c r="G26" t="str">
+        <v>job_title</v>
+      </c>
+      <c r="H26">
+        <v>1</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Analyse de la demande CRM</v>
+      </c>
+      <c r="J26">
+        <v>1</v>
+      </c>
+      <c r="K26" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L26" t="str">
+        <v/>
+      </c>
+      <c r="M26" t="str">
+        <v/>
+      </c>
+      <c r="N26" t="str">
+        <v>none</v>
+      </c>
+      <c r="O26" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P26" t="str">
+        <v>44444444-4444-4444-4444-444444444444</v>
+      </c>
+      <c r="Q26" t="str">
+        <v>221274d2-870c-4b8f-bff0-b49e7f345c7c</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B27" t="str">
+        <v>SUPPORT PIPEDRIVE</v>
+      </c>
+      <c r="C27">
+        <v>4</v>
+      </c>
+      <c r="D27" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="E27" t="str">
+        <v>CHEF DE PROJET DIGITAL</v>
+      </c>
+      <c r="F27" t="str">
+        <v>59297fc0-b709-4908-bdfe-be7c04c0eb46</v>
+      </c>
+      <c r="G27" t="str">
+        <v>job_title</v>
+      </c>
+      <c r="H27">
+        <v>2</v>
+      </c>
+      <c r="I27" t="str">
+        <v>Configuration Pipedrive</v>
+      </c>
+      <c r="J27">
+        <v>2</v>
+      </c>
+      <c r="K27" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L27" t="str">
+        <v/>
+      </c>
+      <c r="M27" t="str">
+        <v/>
+      </c>
+      <c r="N27" t="str">
+        <v>none</v>
+      </c>
+      <c r="O27" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P27" t="str">
+        <v>44444444-4444-4444-4444-444444444444</v>
+      </c>
+      <c r="Q27" t="str">
+        <v>13fcfc07-606c-4d9f-8667-2ad59a8dd6b9</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B28" t="str">
+        <v>SUPPORT PIPEDRIVE</v>
+      </c>
+      <c r="C28">
+        <v>4</v>
+      </c>
+      <c r="D28" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="E28" t="str">
+        <v>CHEF DE PROJET DIGITAL</v>
+      </c>
+      <c r="F28" t="str">
+        <v>59297fc0-b709-4908-bdfe-be7c04c0eb46</v>
+      </c>
+      <c r="G28" t="str">
+        <v>job_title</v>
+      </c>
+      <c r="H28">
+        <v>3</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Formation utilisateur</v>
+      </c>
+      <c r="J28">
+        <v>1</v>
+      </c>
+      <c r="K28" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L28" t="str">
+        <v/>
+      </c>
+      <c r="M28" t="str">
+        <v/>
+      </c>
+      <c r="N28" t="str">
+        <v>none</v>
+      </c>
+      <c r="O28" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P28" t="str">
+        <v>44444444-4444-4444-4444-444444444444</v>
+      </c>
+      <c r="Q28" t="str">
+        <v>b6d9b4a0-d001-4edc-91f1-752b6553b8e5</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B29" t="str">
+        <v>SUPPORT LUCCA</v>
+      </c>
+      <c r="C29">
+        <v>5</v>
+      </c>
+      <c r="D29" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="E29" t="str">
+        <v>CHEF DE PROJET DIGITAL</v>
+      </c>
+      <c r="F29" t="str">
+        <v>59297fc0-b709-4908-bdfe-be7c04c0eb46</v>
+      </c>
+      <c r="G29" t="str">
+        <v>job_title</v>
+      </c>
+      <c r="H29">
+        <v>1</v>
+      </c>
+      <c r="I29" t="str">
+        <v>Analyse de la demande RH</v>
+      </c>
+      <c r="J29">
+        <v>1</v>
+      </c>
+      <c r="K29" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L29" t="str">
+        <v/>
+      </c>
+      <c r="M29" t="str">
+        <v/>
+      </c>
+      <c r="N29" t="str">
+        <v>none</v>
+      </c>
+      <c r="O29" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P29" t="str">
+        <v>55555555-5555-5555-5555-555555555555</v>
+      </c>
+      <c r="Q29" t="str">
+        <v>9f8c965a-8cd6-4abc-8027-2c596b642e4a</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B30" t="str">
+        <v>SUPPORT LUCCA</v>
+      </c>
+      <c r="C30">
+        <v>5</v>
+      </c>
+      <c r="D30" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="E30" t="str">
+        <v>CHEF DE PROJET DIGITAL</v>
+      </c>
+      <c r="F30" t="str">
+        <v>59297fc0-b709-4908-bdfe-be7c04c0eb46</v>
+      </c>
+      <c r="G30" t="str">
+        <v>job_title</v>
+      </c>
+      <c r="H30">
+        <v>2</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Intervention sur Lucca</v>
+      </c>
+      <c r="J30">
+        <v>2</v>
+      </c>
+      <c r="K30" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L30" t="str">
+        <v/>
+      </c>
+      <c r="M30" t="str">
+        <v/>
+      </c>
+      <c r="N30" t="str">
+        <v>none</v>
+      </c>
+      <c r="O30" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P30" t="str">
+        <v>55555555-5555-5555-5555-555555555555</v>
+      </c>
+      <c r="Q30" t="str">
+        <v>d962875c-d9cc-4419-9146-124919996fd9</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B31" t="str">
+        <v>SUPPORT LUCCA</v>
+      </c>
+      <c r="C31">
+        <v>5</v>
+      </c>
+      <c r="D31" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="E31" t="str">
+        <v>CHEF DE PROJET DIGITAL</v>
+      </c>
+      <c r="F31" t="str">
+        <v>59297fc0-b709-4908-bdfe-be7c04c0eb46</v>
+      </c>
+      <c r="G31" t="str">
+        <v>job_title</v>
+      </c>
+      <c r="H31">
+        <v>3</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Validation RH</v>
+      </c>
+      <c r="J31">
+        <v>1</v>
+      </c>
+      <c r="K31" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L31" t="str">
+        <v/>
+      </c>
+      <c r="M31" t="str">
+        <v/>
+      </c>
+      <c r="N31" t="str">
+        <v>none</v>
+      </c>
+      <c r="O31" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P31" t="str">
+        <v>55555555-5555-5555-5555-555555555555</v>
+      </c>
+      <c r="Q31" t="str">
+        <v>0c33d6bf-0638-4633-bccb-670ebbbcba75</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B32" t="str">
+        <v>DEMANDE D'INTERVENTION IT</v>
+      </c>
+      <c r="C32">
+        <v>6</v>
+      </c>
+      <c r="D32" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="E32" t="str">
+        <v>TECHNICIEN IT</v>
+      </c>
+      <c r="F32" t="str">
+        <v>640b7ff1-df57-4bab-a287-67f04a3c4f1e</v>
+      </c>
+      <c r="G32" t="str">
+        <v>job_title</v>
+      </c>
+      <c r="H32">
+        <v>0</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Intervention directe</v>
+      </c>
+      <c r="J32">
+        <v>7</v>
+      </c>
+      <c r="K32" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L32" t="str">
+        <v/>
+      </c>
+      <c r="M32" t="str">
+        <v/>
+      </c>
+      <c r="N32" t="str">
+        <v>none</v>
+      </c>
+      <c r="O32" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P32" t="str">
+        <v>10a38748-7145-4368-821d-03a36924830d</v>
+      </c>
+      <c r="Q32" t="str">
+        <v>5415a2e4-6236-4605-9240-bbf5e9d00e0b</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B33" t="str">
+        <v>DEMANDE D'INTERVENTION IT</v>
+      </c>
+      <c r="C33">
+        <v>6</v>
+      </c>
+      <c r="D33" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="E33" t="str">
+        <v>TECHNICIEN IT</v>
+      </c>
+      <c r="F33" t="str">
+        <v>640b7ff1-df57-4bab-a287-67f04a3c4f1e</v>
+      </c>
+      <c r="G33" t="str">
+        <v>job_title</v>
+      </c>
+      <c r="H33">
+        <v>1</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Ouverture ticket chez Nirwana</v>
+      </c>
+      <c r="J33">
+        <v>1</v>
+      </c>
+      <c r="K33" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L33" t="str">
+        <v/>
+      </c>
+      <c r="M33" t="str">
+        <v/>
+      </c>
+      <c r="N33" t="str">
+        <v>none</v>
+      </c>
+      <c r="O33" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P33" t="str">
+        <v>10a38748-7145-4368-821d-03a36924830d</v>
+      </c>
+      <c r="Q33" t="str">
+        <v>1165f076-f6d3-492b-85ee-8093756267e7</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B34" t="str">
+        <v>REPORTING POWER BI</v>
+      </c>
+      <c r="C34">
+        <v>6</v>
+      </c>
+      <c r="D34" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="E34" t="str">
+        <v>CHEF DE PROJET DIGITAL</v>
+      </c>
+      <c r="F34" t="str">
+        <v>59297fc0-b709-4908-bdfe-be7c04c0eb46</v>
+      </c>
+      <c r="G34" t="str">
+        <v>job_title</v>
+      </c>
+      <c r="H34">
+        <v>1</v>
+      </c>
+      <c r="I34" t="str">
+        <v>Analyse des besoins reporting</v>
+      </c>
+      <c r="J34">
+        <v>1</v>
+      </c>
+      <c r="K34" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L34" t="str">
+        <v/>
+      </c>
+      <c r="M34" t="str">
+        <v/>
+      </c>
+      <c r="N34" t="str">
+        <v>none</v>
+      </c>
+      <c r="O34" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P34" t="str">
+        <v>66666666-6666-6666-6666-666666666666</v>
+      </c>
+      <c r="Q34" t="str">
+        <v>dc69375e-02a3-4d39-9b08-f34776e66be3</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B35" t="str">
+        <v>REPORTING POWER BI</v>
+      </c>
+      <c r="C35">
+        <v>6</v>
+      </c>
+      <c r="D35" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="E35" t="str">
+        <v>CHEF DE PROJET DIGITAL</v>
+      </c>
+      <c r="F35" t="str">
+        <v>59297fc0-b709-4908-bdfe-be7c04c0eb46</v>
+      </c>
+      <c r="G35" t="str">
+        <v>job_title</v>
+      </c>
+      <c r="H35">
+        <v>2</v>
+      </c>
+      <c r="I35" t="str">
+        <v>Développement du rapport</v>
+      </c>
+      <c r="J35">
+        <v>5</v>
+      </c>
+      <c r="K35" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L35" t="str">
+        <v/>
+      </c>
+      <c r="M35" t="str">
+        <v/>
+      </c>
+      <c r="N35" t="str">
+        <v>none</v>
+      </c>
+      <c r="O35" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P35" t="str">
+        <v>66666666-6666-6666-6666-666666666666</v>
+      </c>
+      <c r="Q35" t="str">
+        <v>e65a6811-afa4-460e-b8ba-b763dd910a7f</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B36" t="str">
+        <v>REPORTING POWER BI</v>
+      </c>
+      <c r="C36">
+        <v>6</v>
+      </c>
+      <c r="D36" t="str">
+        <v>fixed_role</v>
+      </c>
+      <c r="E36" t="str">
+        <v>CHEF DE PROJET DIGITAL</v>
+      </c>
+      <c r="F36" t="str">
+        <v>59297fc0-b709-4908-bdfe-be7c04c0eb46</v>
+      </c>
+      <c r="G36" t="str">
+        <v>job_title</v>
+      </c>
+      <c r="H36">
+        <v>3</v>
+      </c>
+      <c r="I36" t="str">
+        <v>Tests et publication</v>
+      </c>
+      <c r="J36">
+        <v>2</v>
+      </c>
+      <c r="K36" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L36" t="str">
+        <v/>
+      </c>
+      <c r="M36" t="str">
+        <v/>
+      </c>
+      <c r="N36" t="str">
+        <v>none</v>
+      </c>
+      <c r="O36" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P36" t="str">
+        <v>66666666-6666-6666-6666-666666666666</v>
+      </c>
+      <c r="Q36" t="str">
+        <v>725c1af3-dfe2-43e7-973f-7ef25bfcf0a0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B37" t="str">
+        <v>SUPPORT MATERIEL BUREAUTIQUE</v>
+      </c>
+      <c r="C37">
+        <v>7</v>
+      </c>
+      <c r="D37" t="str">
+        <v>manager_dispatch</v>
+      </c>
+      <c r="E37" t="str">
+        <v>SG</v>
+      </c>
+      <c r="F37" t="str">
+        <v>bf2b99fc-eec9-44f2-9738-a5b23d9bee11</v>
+      </c>
+      <c r="G37" t="str">
+        <v>department</v>
+      </c>
+      <c r="H37">
+        <v>1</v>
+      </c>
+      <c r="I37" t="str">
+        <v>Diagnostic matériel</v>
+      </c>
+      <c r="J37">
+        <v>1</v>
+      </c>
+      <c r="K37" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L37" t="str">
+        <v/>
+      </c>
+      <c r="M37" t="str">
+        <v/>
+      </c>
+      <c r="N37" t="str">
+        <v>none</v>
+      </c>
+      <c r="O37" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P37" t="str">
+        <v>77777777-7777-7777-7777-777777777777</v>
+      </c>
+      <c r="Q37" t="str">
+        <v>4693ec6a-4761-4c09-820b-d85cf5e71a63</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B38" t="str">
+        <v>SUPPORT MATERIEL BUREAUTIQUE</v>
+      </c>
+      <c r="C38">
+        <v>7</v>
+      </c>
+      <c r="D38" t="str">
+        <v>manager_dispatch</v>
+      </c>
+      <c r="E38" t="str">
+        <v>SG</v>
+      </c>
+      <c r="F38" t="str">
+        <v>bf2b99fc-eec9-44f2-9738-a5b23d9bee11</v>
+      </c>
+      <c r="G38" t="str">
+        <v>department</v>
+      </c>
+      <c r="H38">
+        <v>2</v>
+      </c>
+      <c r="I38" t="str">
+        <v>Commande / Remplacement</v>
+      </c>
+      <c r="J38">
+        <v>3</v>
+      </c>
+      <c r="K38" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L38" t="str">
+        <v/>
+      </c>
+      <c r="M38" t="str">
+        <v/>
+      </c>
+      <c r="N38" t="str">
+        <v>none</v>
+      </c>
+      <c r="O38" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P38" t="str">
+        <v>77777777-7777-7777-7777-777777777777</v>
+      </c>
+      <c r="Q38" t="str">
+        <v>68ac3914-f166-4263-9219-ae286ae5fa7d</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B39" t="str">
+        <v>SUPPORT MATERIEL BUREAUTIQUE</v>
+      </c>
+      <c r="C39">
+        <v>7</v>
+      </c>
+      <c r="D39" t="str">
+        <v>manager_dispatch</v>
+      </c>
+      <c r="E39" t="str">
+        <v>SG</v>
+      </c>
+      <c r="F39" t="str">
+        <v>bf2b99fc-eec9-44f2-9738-a5b23d9bee11</v>
+      </c>
+      <c r="G39" t="str">
+        <v>department</v>
+      </c>
+      <c r="H39">
+        <v>3</v>
+      </c>
+      <c r="I39" t="str">
+        <v>Installation et configuration</v>
+      </c>
+      <c r="J39">
+        <v>2</v>
+      </c>
+      <c r="K39" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L39" t="str">
+        <v/>
+      </c>
+      <c r="M39" t="str">
+        <v/>
+      </c>
+      <c r="N39" t="str">
+        <v>none</v>
+      </c>
+      <c r="O39" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P39" t="str">
+        <v>77777777-7777-7777-7777-777777777777</v>
+      </c>
+      <c r="Q39" t="str">
+        <v>b8a1664a-9e58-4eca-a92c-d9c2560246b0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B40" t="str">
+        <v>SUPPORT MATERIEL BUREAUTIQUE</v>
+      </c>
+      <c r="C40">
+        <v>7</v>
+      </c>
+      <c r="D40" t="str">
+        <v>manager_dispatch</v>
+      </c>
+      <c r="E40" t="str">
+        <v>SG</v>
+      </c>
+      <c r="F40" t="str">
+        <v>bf2b99fc-eec9-44f2-9738-a5b23d9bee11</v>
+      </c>
+      <c r="G40" t="str">
+        <v>department</v>
+      </c>
+      <c r="H40">
+        <v>4</v>
+      </c>
+      <c r="I40" t="str">
+        <v>Validation utilisateur</v>
+      </c>
+      <c r="J40">
+        <v>1</v>
+      </c>
+      <c r="K40" t="str">
+        <v>parallel</v>
+      </c>
+      <c r="L40" t="str">
+        <v/>
+      </c>
+      <c r="M40" t="str">
+        <v/>
+      </c>
+      <c r="N40" t="str">
+        <v>none</v>
+      </c>
+      <c r="O40" t="str">
+        <v>47b00c1b-e2a7-4b89-a1ed-a827057b0f8e</v>
+      </c>
+      <c r="P40" t="str">
+        <v>77777777-7777-7777-7777-777777777777</v>
+      </c>
+      <c r="Q40" t="str">
+        <v>a6491c6f-f917-4ecb-a51f-331267019999</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q40"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I8"/>
+  <cols>
+    <col min="1" max="1" width="40.83203125" customWidth="1"/>
+    <col min="2" max="2" width="42.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
+    <col min="5" max="5" width="34.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID_processus</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Processus</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Code</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Libellé</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Couleur</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Ordre</v>
+      </c>
+      <c r="G1" t="str">
+        <v>État initial</v>
+      </c>
+      <c r="H1" t="str">
+        <v>État final</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Catégorie</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v>soumise</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Soumise</v>
+      </c>
+      <c r="E2" t="str">
+        <v>bg-slate-100 text-slate-700</v>
+      </c>
+      <c r="F2">
+        <v>10</v>
+      </c>
+      <c r="G2" t="str">
+        <v>oui</v>
+      </c>
+      <c r="H2" t="str">
+        <v>non</v>
+      </c>
+      <c r="I2" t="str">
+        <v>SOUMIS</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v/>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v>en_cours</v>
+      </c>
+      <c r="D3" t="str">
+        <v>En cours</v>
+      </c>
+      <c r="E3" t="str">
+        <v>bg-amber-100 text-amber-700</v>
+      </c>
+      <c r="F3">
+        <v>20</v>
+      </c>
+      <c r="G3" t="str">
+        <v>non</v>
+      </c>
+      <c r="H3" t="str">
+        <v>non</v>
+      </c>
+      <c r="I3" t="str">
+        <v>EN_COURS</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v/>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v>a_valider</v>
+      </c>
+      <c r="D4" t="str">
+        <v>À valider</v>
+      </c>
+      <c r="E4" t="str">
+        <v>bg-violet-100 text-violet-700</v>
+      </c>
+      <c r="F4">
+        <v>30</v>
+      </c>
+      <c r="G4" t="str">
+        <v>non</v>
+      </c>
+      <c r="H4" t="str">
+        <v>non</v>
+      </c>
+      <c r="I4" t="str">
+        <v>EN_ATTENTE_VALIDATION</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v>validee</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Validée</v>
+      </c>
+      <c r="E5" t="str">
+        <v>bg-emerald-100 text-emerald-700</v>
+      </c>
+      <c r="F5">
+        <v>40</v>
+      </c>
+      <c r="G5" t="str">
+        <v>non</v>
+      </c>
+      <c r="H5" t="str">
+        <v>non</v>
+      </c>
+      <c r="I5" t="str">
+        <v>EN_COURS</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v/>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v>terminee</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Terminée</v>
+      </c>
+      <c r="E6" t="str">
+        <v>bg-emerald-200 text-emerald-800</v>
+      </c>
+      <c r="F6">
+        <v>50</v>
+      </c>
+      <c r="G6" t="str">
+        <v>non</v>
+      </c>
+      <c r="H6" t="str">
+        <v>oui</v>
+      </c>
+      <c r="I6" t="str">
+        <v>TERMINE</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v>refusee</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Refusée</v>
+      </c>
+      <c r="E7" t="str">
+        <v>bg-red-100 text-red-700</v>
+      </c>
+      <c r="F7">
+        <v>60</v>
+      </c>
+      <c r="G7" t="str">
+        <v>non</v>
+      </c>
+      <c r="H7" t="str">
+        <v>oui</v>
+      </c>
+      <c r="I7" t="str">
+        <v>TERMINE</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v/>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v>annulee</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Annulée</v>
+      </c>
+      <c r="E8" t="str">
+        <v>bg-red-100 text-red-700</v>
+      </c>
+      <c r="F8">
+        <v>70</v>
+      </c>
+      <c r="G8" t="str">
+        <v>non</v>
+      </c>
+      <c r="H8" t="str">
+        <v>oui</v>
+      </c>
+      <c r="I8" t="str">
+        <v>TERMINE</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:I8"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A54"/>
+  <cols>
+    <col min="1" max="1" width="115.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>🛠  Paramétrage en masse — Autres flux</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>ONGLETS :</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v xml:space="preserve">  0. EXISTANT             — DUMP READ-ONLY de tous les flux configurés actuellement en DB (hors BE)</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v xml:space="preserve">                            32 lignes : COMPTABILITÉ, GESTION REGLEMENTAIRE, Innovation, ONBOARDING,</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v xml:space="preserve">                            QUALITÉ SECURITE ENVIRONNEMENT, SERVICE ACHAT, SERVICE MAINTENANCE,</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v xml:space="preserve">                            SERVICE MARKETING, SUPPORT IT/DIGITAL (avec ses 6 sous-processus)</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v xml:space="preserve">  0bis. TABLE_EFFECTS     — effets de bord sur tables métier (supplier_waiting_approval,</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v xml:space="preserve">                            suppliers, nc_declarations, nc_actions, inno_demandes, demande_materiel)</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v xml:space="preserve">                            → permet de voir quelles étapes déclenchent une INSERT/UPDATE sur quelle table</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v xml:space="preserve">  1. SERVICE_ACHAT        — étapes existantes du flux Achat (à compléter)</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v xml:space="preserve">  2. NOUVELLES_ETAPES     — saisie des étapes IT / RH / Comm / Maintenance / Logistique / Innovation</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v xml:space="preserve">  3. PROCESS_REFERENCE    — UUID des process à utiliser dans la colonne ID_processus</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v xml:space="preserve">  4. PROFILES_REFERENCE   — UUID des utilisateurs (pour Affectation cible (UUID) quand type=fixed_user/manager_dispatch)</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v xml:space="preserve">  5. DEPARTMENTS_REFERENCE— UUID des départements (pour Affectation cible (UUID) quand type=department)</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v xml:space="preserve">  6. GROUPS_REFERENCE     — UUID des groupes collaborateurs (pour Affectation cible (UUID) quand type=group)</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v xml:space="preserve">  7. ASSIGNMENT_TYPES     — cheat-sheet des 7 modes d'affectation supportés</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v xml:space="preserve">  8. ETATS_PAR_FLUX       — liste des états par processus + colonne Catégorie macro</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>⚠ AFFECTATION — 2 cas à distinguer :</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v xml:space="preserve">  CAS A — toutes les étapes d'un sous-processus → MÊME affectataire :</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v xml:space="preserve">     Remplis Affectation type/cible UNIQUEMENT sur la ligne N°=1.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v xml:space="preserve">     → Je génère un sub_process_templates classique (affectation au niveau sous-processus).</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v xml:space="preserve">  CAS B — chaque étape a un affectataire DIFFÉRENT (ex: Achat puis Comptabilité) :</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v xml:space="preserve">     Remplis Affectation type/cible sur CHAQUE ligne (N°=1, 2, 3…).</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v xml:space="preserve">     → Je génère un workflow state-machine (wf_workflows/wf_steps), comme le flux</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v xml:space="preserve">       « Demande de nouveau fournisseur » qui passe : Vérification (groupe Achat) →</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v xml:space="preserve">       Création (groupe Comptabilité) → Terminé.</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v xml:space="preserve">  Pour les types « requester » et « manager_requester », laisse UUID vide.</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v xml:space="preserve">  Pour « fixed_user » / « manager_dispatch » : colle l'UUID depuis PROFILES_REFERENCE.</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v xml:space="preserve">  Pour « department » : colle l'UUID depuis DEPARTMENTS_REFERENCE.</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v xml:space="preserve">  Pour « group » : colle l'UUID depuis GROUPS_REFERENCE.</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>POUR SAISIR DES ÉTAPES SUR UN FLUX SANS ÉTAPES (ex: IT - Demande d'intervention IT) :</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v xml:space="preserve">  1. Va sur PROCESS_REFERENCE → copie l'ID_processus du flux concerné</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v xml:space="preserve">  2. Va sur NOUVELLES_ETAPES → colle l'ID dans ID_processus + nom dans Processus</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v xml:space="preserve">  3. Définis ID_sous_processus (UUID que tu inventes, format xxxxxxxx-xxxx-xxxx-xxxx-xxxxxxxxxxxx) +</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v xml:space="preserve">     Sous-processus (nom). Tu peux créer plusieurs sous-processus par flux.</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v xml:space="preserve">  4. Pour chaque sous-processus, ajoute autant de lignes que d'étapes (N° 1, 2, 3…)</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v xml:space="preserve">  5. Sur la ligne N°=1 du sous-processus, renseigne les colonnes Affectation</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>POUR DÉFINIR LES ÉTATS D'UN FLUX :</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v xml:space="preserve">  → ETATS_PAR_FLUX : recopie le bloc des 7 lignes par flux, ajuste si besoin.</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v xml:space="preserve">  → Catégorie : SOUMIS | EN_COURS | EN_ATTENTE_VALIDATION | EN_ATTENTE_RETOUR_ADMIN | EN_ATTENTE_TRAVAUX | TERMINE</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>QUAND C'EST PRÊT :</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v xml:space="preserve">  Renvoie ce fichier à Claude — il génèrera :</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v xml:space="preserve">     • UPSERT sub_process_templates (assignment_type + target_*)</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v xml:space="preserve">     • INSERT task_templates (étapes + output_state_code)</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v xml:space="preserve">     • INSERT request_states (avec catégorie macro)</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v xml:space="preserve">  Backup automatique avant écriture, comme pour le BE.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:A54"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G13"/>
+  <cols>
+    <col min="1" max="1" width="32.83203125" customWidth="1"/>
+    <col min="2" max="2" width="48.83203125" customWidth="1"/>
+    <col min="3" max="3" width="42.83203125" customWidth="1"/>
+    <col min="4" max="4" width="34.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="60.83203125" customWidth="1"/>
+    <col min="7" max="7" width="80.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Processus</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Sous-processus</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Étape concernée</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Table impactée</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Action</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Champs copiés</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>SERVICE ACHAT</v>
+      </c>
+      <c r="B2" t="str">
+        <v>DEMANDE DE NOUVEAU FOURNISSEUR</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Soumission formulaire</v>
+      </c>
+      <c r="D2" t="str">
+        <v>supplier_waiting_approval</v>
+      </c>
+      <c r="E2" t="str">
+        <v>INSERT (status='a_completer')</v>
+      </c>
+      <c r="F2" t="str">
+        <v>siret, tva, raison_sociale, ca_estime, contacts (nom/email/tel/poste), famille, pièces jointes (RIB, KBIS)</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Géré directement par NewSupplierRequestDialog.tsx (pas de tasks)</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>SERVICE ACHAT</v>
+      </c>
+      <c r="B3" t="str">
+        <v>DEMANDE DE NOUVEAU FOURNISSEUR</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Tâche 1 — Vérification fournisseur (Groupe Service Achat)</v>
+      </c>
+      <c r="D3" t="str">
+        <v>supplier_waiting_approval</v>
+      </c>
+      <c r="E3" t="str">
+        <v>UPDATE (status='validee' ou 'a_completer' si refus)</v>
+      </c>
+      <c r="F3" t="str">
+        <v>completeness_score, validated_by, validated_at, refusal_reason</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Workflow porté par tâche d1111111. Si refus → demandeur complète.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>SERVICE ACHAT</v>
+      </c>
+      <c r="B4" t="str">
+        <v>DEMANDE DE NOUVEAU FOURNISSEUR</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Tâche 2 — Création fournisseur (Groupe Comptabilité)</v>
+      </c>
+      <c r="D4" t="str">
+        <v>suppliers (création)</v>
+      </c>
+      <c r="E4" t="str">
+        <v>INSERT depuis supplier_waiting_approval</v>
+      </c>
+      <c r="F4" t="str">
+        <v>numero_fournisseur (saisi), + recopie des champs de supplier_waiting_approval</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Tâche d2222222 → la Compta saisit le numero Divalto, copie dans suppliers, supprime/archive de supplier_waiting_approval.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>QUALITÉ SECURITE ENVIRONNEMENT</v>
+      </c>
+      <c r="B5" t="str">
+        <v>DECLARATION DE NON CONFORMITE</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Soumission formulaire</v>
+      </c>
+      <c r="D5" t="str">
+        <v>nc_declarations</v>
+      </c>
+      <c r="E5" t="str">
+        <v>INSERT (status='soumise')</v>
+      </c>
+      <c r="F5" t="str">
+        <v>type, gravite, description, site, pilote, pieces jointes</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Géré par SMQNewDeclaration.tsx — pas via tasks. Workflow ensuite via nc_actions / nc_status_history.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>QUALITÉ SECURITE ENVIRONNEMENT</v>
+      </c>
+      <c r="B6" t="str">
+        <v>DECLARATION DE NON CONFORMITE</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Actions correctives / préventives</v>
+      </c>
+      <c r="D6" t="str">
+        <v>nc_actions</v>
+      </c>
+      <c r="E6" t="str">
+        <v>INSERT par étape</v>
+      </c>
+      <c r="F6" t="str">
+        <v>description action, responsable, échéance, statut</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Multi-actions par déclaration. Pilote NC géré via nc_process_pilots.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Innovation</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Demande Innovation</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Soumission formulaire</v>
+      </c>
+      <c r="D7" t="str">
+        <v>inno_demandes</v>
+      </c>
+      <c r="E7" t="str">
+        <v>INSERT</v>
+      </c>
+      <c r="F7" t="str">
+        <v>titre, description, code_projet, étiquettes (suggestions auto), usage</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Géré par InnovationNew.tsx. Tâches générées en parallèle (Instruire, CODIR, Mettre en oeuvre).</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>SERVICE MAINTENANCE</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Demande de matériel</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Soumission formulaire</v>
+      </c>
+      <c r="D8" t="str">
+        <v>demande_materiel</v>
+      </c>
+      <c r="E8" t="str">
+        <v>INSERT</v>
+      </c>
+      <c r="F8" t="str">
+        <v>site, équipement, urgence, description, pieces jointes</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Géré par NewMaintenanceRequest.tsx. Tâche unique de traitement assignée.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>SUPPORT IT/DIGITAL</v>
+      </c>
+      <c r="B9" t="str">
+        <v>(tous sous-processus)</v>
+      </c>
+      <c r="C9" t="str">
+        <v>—</v>
+      </c>
+      <c r="D9" t="str">
+        <v>(aucune table dédiée)</v>
+      </c>
+      <c r="E9" t="str">
+        <v>—</v>
+      </c>
+      <c r="F9" t="str">
+        <v>—</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Flux 100% tasks — pas d'effet de bord sur table métier dédiée.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>GESTION REGLEMENTAIRE</v>
+      </c>
+      <c r="B10" t="str">
+        <v>RAPPORT ANNUEL ICPE / RED3</v>
+      </c>
+      <c r="C10" t="str">
+        <v>—</v>
+      </c>
+      <c r="D10" t="str">
+        <v>(aucune table dédiée)</v>
+      </c>
+      <c r="E10" t="str">
+        <v>—</v>
+      </c>
+      <c r="F10" t="str">
+        <v>—</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Flux 100% tasks, pilotées par le Manager Exploitation Keon.bio.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>ONBOARDING</v>
+      </c>
+      <c r="B11" t="str">
+        <v>ONBOARDING / MUTATION / OFFBOARDING / PROMOTION</v>
+      </c>
+      <c r="C11" t="str">
+        <v>—</v>
+      </c>
+      <c r="D11" t="str">
+        <v>(aucune table dédiée)</v>
+      </c>
+      <c r="E11" t="str">
+        <v>—</v>
+      </c>
+      <c r="F11" t="str">
+        <v>—</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Tâches IT only (pas de table RH dédiée).</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>SERVICE MARKETING</v>
+      </c>
+      <c r="B12" t="str">
+        <v>RESERVATION DES STANDS POUR LES SALONS</v>
+      </c>
+      <c r="C12" t="str">
+        <v>—</v>
+      </c>
+      <c r="D12" t="str">
+        <v>(aucune table dédiée)</v>
+      </c>
+      <c r="E12" t="str">
+        <v>—</v>
+      </c>
+      <c r="F12" t="str">
+        <v>—</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Flux 100% tasks.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>COMPTABILITÉ</v>
+      </c>
+      <c r="B13" t="str">
+        <v>AJOUT DE CLIENT</v>
+      </c>
+      <c r="C13" t="str">
+        <v>—</v>
+      </c>
+      <c r="D13" t="str">
+        <v>(table clients à créer ?)</v>
+      </c>
+      <c r="E13" t="str">
+        <v>—</v>
+      </c>
+      <c r="F13" t="str">
+        <v>—</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Pas de table 'clients' dédiée pour l'instant — uniquement tâche de création. Possible évolution future à l'image de supplier_waiting_approval.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G13"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Q4"/>
   <cols>
     <col min="1" max="1" width="38.83203125" customWidth="1"/>
@@ -645,7 +3629,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:R9"/>
   <cols>
@@ -1180,7 +4164,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B21"/>
   <cols>
@@ -1363,7 +4347,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D103"/>
   <cols>
@@ -2822,7 +5806,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B63"/>
   <cols>
@@ -3341,7 +6325,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D6"/>
   <cols>
@@ -3442,7 +6426,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B8"/>
   <cols>
@@ -3519,482 +6503,4 @@
     <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
   </ignoredErrors>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I8"/>
-  <cols>
-    <col min="1" max="1" width="40.83203125" customWidth="1"/>
-    <col min="2" max="2" width="42.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
-    <col min="5" max="5" width="34.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>ID_processus</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Processus</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Code</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Libellé</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Couleur</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Ordre</v>
-      </c>
-      <c r="G1" t="str">
-        <v>État initial</v>
-      </c>
-      <c r="H1" t="str">
-        <v>État final</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Catégorie</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v/>
-      </c>
-      <c r="B2" t="str">
-        <v/>
-      </c>
-      <c r="C2" t="str">
-        <v>soumise</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Soumise</v>
-      </c>
-      <c r="E2" t="str">
-        <v>bg-slate-100 text-slate-700</v>
-      </c>
-      <c r="F2">
-        <v>10</v>
-      </c>
-      <c r="G2" t="str">
-        <v>oui</v>
-      </c>
-      <c r="H2" t="str">
-        <v>non</v>
-      </c>
-      <c r="I2" t="str">
-        <v>SOUMIS</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v/>
-      </c>
-      <c r="B3" t="str">
-        <v/>
-      </c>
-      <c r="C3" t="str">
-        <v>en_cours</v>
-      </c>
-      <c r="D3" t="str">
-        <v>En cours</v>
-      </c>
-      <c r="E3" t="str">
-        <v>bg-amber-100 text-amber-700</v>
-      </c>
-      <c r="F3">
-        <v>20</v>
-      </c>
-      <c r="G3" t="str">
-        <v>non</v>
-      </c>
-      <c r="H3" t="str">
-        <v>non</v>
-      </c>
-      <c r="I3" t="str">
-        <v>EN_COURS</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v/>
-      </c>
-      <c r="B4" t="str">
-        <v/>
-      </c>
-      <c r="C4" t="str">
-        <v>a_valider</v>
-      </c>
-      <c r="D4" t="str">
-        <v>À valider</v>
-      </c>
-      <c r="E4" t="str">
-        <v>bg-violet-100 text-violet-700</v>
-      </c>
-      <c r="F4">
-        <v>30</v>
-      </c>
-      <c r="G4" t="str">
-        <v>non</v>
-      </c>
-      <c r="H4" t="str">
-        <v>non</v>
-      </c>
-      <c r="I4" t="str">
-        <v>EN_ATTENTE_VALIDATION</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v/>
-      </c>
-      <c r="B5" t="str">
-        <v/>
-      </c>
-      <c r="C5" t="str">
-        <v>validee</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Validée</v>
-      </c>
-      <c r="E5" t="str">
-        <v>bg-emerald-100 text-emerald-700</v>
-      </c>
-      <c r="F5">
-        <v>40</v>
-      </c>
-      <c r="G5" t="str">
-        <v>non</v>
-      </c>
-      <c r="H5" t="str">
-        <v>non</v>
-      </c>
-      <c r="I5" t="str">
-        <v>EN_COURS</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v/>
-      </c>
-      <c r="B6" t="str">
-        <v/>
-      </c>
-      <c r="C6" t="str">
-        <v>terminee</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Terminée</v>
-      </c>
-      <c r="E6" t="str">
-        <v>bg-emerald-200 text-emerald-800</v>
-      </c>
-      <c r="F6">
-        <v>50</v>
-      </c>
-      <c r="G6" t="str">
-        <v>non</v>
-      </c>
-      <c r="H6" t="str">
-        <v>oui</v>
-      </c>
-      <c r="I6" t="str">
-        <v>TERMINE</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v/>
-      </c>
-      <c r="B7" t="str">
-        <v/>
-      </c>
-      <c r="C7" t="str">
-        <v>refusee</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Refusée</v>
-      </c>
-      <c r="E7" t="str">
-        <v>bg-red-100 text-red-700</v>
-      </c>
-      <c r="F7">
-        <v>60</v>
-      </c>
-      <c r="G7" t="str">
-        <v>non</v>
-      </c>
-      <c r="H7" t="str">
-        <v>oui</v>
-      </c>
-      <c r="I7" t="str">
-        <v>TERMINE</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v/>
-      </c>
-      <c r="B8" t="str">
-        <v/>
-      </c>
-      <c r="C8" t="str">
-        <v>annulee</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Annulée</v>
-      </c>
-      <c r="E8" t="str">
-        <v>bg-red-100 text-red-700</v>
-      </c>
-      <c r="F8">
-        <v>70</v>
-      </c>
-      <c r="G8" t="str">
-        <v>non</v>
-      </c>
-      <c r="H8" t="str">
-        <v>oui</v>
-      </c>
-      <c r="I8" t="str">
-        <v>TERMINE</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I8"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A47"/>
-  <cols>
-    <col min="1" max="1" width="115.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>🛠  Paramétrage en masse — Autres flux</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>ONGLETS :</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v xml:space="preserve">  1. SERVICE_ACHAT        — étapes existantes du flux Achat (à compléter)</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v xml:space="preserve">  2. NOUVELLES_ETAPES     — saisie des étapes IT / RH / Comm / Maintenance / Logistique / Innovation</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v xml:space="preserve">  3. PROCESS_REFERENCE    — UUID des process à utiliser dans la colonne ID_processus</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v xml:space="preserve">  4. PROFILES_REFERENCE   — UUID des utilisateurs (pour Affectation cible (UUID) quand type=fixed_user/manager_dispatch)</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v xml:space="preserve">  5. DEPARTMENTS_REFERENCE— UUID des départements (pour Affectation cible (UUID) quand type=department)</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v xml:space="preserve">  6. GROUPS_REFERENCE     — UUID des groupes collaborateurs (pour Affectation cible (UUID) quand type=group)</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v xml:space="preserve">  7. ASSIGNMENT_TYPES     — cheat-sheet des 7 modes d'affectation supportés</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v xml:space="preserve">  8. ETATS_PAR_FLUX       — liste des états par processus + colonne Catégorie macro</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>⚠ AFFECTATION — 2 cas à distinguer :</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v xml:space="preserve">  CAS A — toutes les étapes d'un sous-processus → MÊME affectataire :</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v xml:space="preserve">     Remplis Affectation type/cible UNIQUEMENT sur la ligne N°=1.</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v xml:space="preserve">     → Je génère un sub_process_templates classique (affectation au niveau sous-processus).</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v xml:space="preserve">  CAS B — chaque étape a un affectataire DIFFÉRENT (ex: Achat puis Comptabilité) :</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v xml:space="preserve">     Remplis Affectation type/cible sur CHAQUE ligne (N°=1, 2, 3…).</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v xml:space="preserve">     → Je génère un workflow state-machine (wf_workflows/wf_steps), comme le flux</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v xml:space="preserve">       « Demande de nouveau fournisseur » qui passe : Vérification (groupe Achat) →</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v xml:space="preserve">       Création (groupe Comptabilité) → Terminé.</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v xml:space="preserve">  Pour les types « requester » et « manager_requester », laisse UUID vide.</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v xml:space="preserve">  Pour « fixed_user » / « manager_dispatch » : colle l'UUID depuis PROFILES_REFERENCE.</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v xml:space="preserve">  Pour « department » : colle l'UUID depuis DEPARTMENTS_REFERENCE.</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v xml:space="preserve">  Pour « group » : colle l'UUID depuis GROUPS_REFERENCE.</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>POUR SAISIR DES ÉTAPES SUR UN FLUX SANS ÉTAPES (ex: IT - Demande d'intervention IT) :</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v xml:space="preserve">  1. Va sur PROCESS_REFERENCE → copie l'ID_processus du flux concerné</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v xml:space="preserve">  2. Va sur NOUVELLES_ETAPES → colle l'ID dans ID_processus + nom dans Processus</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v xml:space="preserve">  3. Définis ID_sous_processus (UUID que tu inventes, format xxxxxxxx-xxxx-xxxx-xxxx-xxxxxxxxxxxx) +</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v xml:space="preserve">     Sous-processus (nom). Tu peux créer plusieurs sous-processus par flux.</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v xml:space="preserve">  4. Pour chaque sous-processus, ajoute autant de lignes que d'étapes (N° 1, 2, 3…)</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v xml:space="preserve">  5. Sur la ligne N°=1 du sous-processus, renseigne les colonnes Affectation</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="str">
-        <v>POUR DÉFINIR LES ÉTATS D'UN FLUX :</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
-        <v xml:space="preserve">  → ETATS_PAR_FLUX : recopie le bloc des 7 lignes par flux, ajuste si besoin.</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="str">
-        <v xml:space="preserve">  → Catégorie : SOUMIS | EN_COURS | EN_ATTENTE_VALIDATION | EN_ATTENTE_RETOUR_ADMIN | EN_ATTENTE_TRAVAUX | TERMINE</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="str">
-        <v>QUAND C'EST PRÊT :</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="str">
-        <v xml:space="preserve">  Renvoie ce fichier à Claude — il génèrera :</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="str">
-        <v xml:space="preserve">     • UPSERT sub_process_templates (assignment_type + target_*)</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="str">
-        <v xml:space="preserve">     • INSERT task_templates (étapes + output_state_code)</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="str">
-        <v xml:space="preserve">     • INSERT request_states (avec catégorie macro)</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="str">
-        <v xml:space="preserve">  Backup automatique avant écriture, comme pour le BE.</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A47"/>
-  </ignoredErrors>
-</worksheet>
 </file>
</xml_diff>